<commit_message>
updated the post-process so it can handle the NA basin as well
</commit_message>
<xml_diff>
--- a/models/resnet18/data_train_statistics.xlsx
+++ b/models/resnet18/data_train_statistics.xlsx
@@ -485,25 +485,25 @@
         <v>0</v>
       </c>
       <c r="C2" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D2" t="n">
-        <v>57244.16796875</v>
+        <v>57229.859375</v>
       </c>
       <c r="E2" t="n">
-        <v>104155.375</v>
+        <v>104148.953125</v>
       </c>
       <c r="F2" t="n">
-        <v>1010045075649.812</v>
+        <v>997938280727.6406</v>
       </c>
       <c r="G2" t="n">
-        <v>100738.3266843829</v>
+        <v>100756.5061103958</v>
       </c>
       <c r="H2" t="n">
-        <v>7189362.991270711</v>
+        <v>6872947.682027092</v>
       </c>
       <c r="I2" t="n">
-        <v>2681.298750842716</v>
+        <v>2621.630729532115</v>
       </c>
     </row>
     <row r="3">
@@ -516,25 +516,25 @@
         <v>0</v>
       </c>
       <c r="C3" t="n">
-        <v>7751633</v>
+        <v>7665278</v>
       </c>
       <c r="D3" t="n">
-        <v>272.838134765625</v>
+        <v>273.029052734375</v>
       </c>
       <c r="E3" t="n">
-        <v>307.6376953125</v>
+        <v>307.64306640625</v>
       </c>
       <c r="F3" t="n">
-        <v>2324946528.585205</v>
+        <v>2299262388.786377</v>
       </c>
       <c r="G3" t="n">
-        <v>299.9299023296387</v>
+        <v>299.9581213866445</v>
       </c>
       <c r="H3" t="n">
-        <v>6.173281914396444</v>
+        <v>6.045553630239024</v>
       </c>
       <c r="I3" t="n">
-        <v>2.484609006342133</v>
+        <v>2.458770755934563</v>
       </c>
     </row>
     <row r="4">
@@ -547,25 +547,25 @@
         <v>1000</v>
       </c>
       <c r="C4" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D4" t="n">
-        <v>-4322.37109375</v>
+        <v>-5028.0546875</v>
       </c>
       <c r="E4" t="n">
-        <v>3362.25</v>
+        <v>3345.8203125</v>
       </c>
       <c r="F4" t="n">
-        <v>13020649555.28638</v>
+        <v>12890629541.0498</v>
       </c>
       <c r="G4" t="n">
-        <v>1298.633576030693</v>
+        <v>1301.498117872192</v>
       </c>
       <c r="H4" t="n">
-        <v>130661.1472207419</v>
+        <v>129566.1263183947</v>
       </c>
       <c r="I4" t="n">
-        <v>361.4708110217779</v>
+        <v>359.9529501454249</v>
       </c>
     </row>
     <row r="5">
@@ -578,25 +578,25 @@
         <v>975</v>
       </c>
       <c r="C5" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D5" t="n">
-        <v>-2161.78466796875</v>
+        <v>-2872.02001953125</v>
       </c>
       <c r="E5" t="n">
-        <v>5434.396484375</v>
+        <v>5412.08740234375</v>
       </c>
       <c r="F5" t="n">
-        <v>34770480594.78125</v>
+        <v>34377225323.5813</v>
       </c>
       <c r="G5" t="n">
-        <v>3467.884867293271</v>
+        <v>3470.885104085111</v>
       </c>
       <c r="H5" t="n">
-        <v>125153.9994691315</v>
+        <v>124054.0283873549</v>
       </c>
       <c r="I5" t="n">
-        <v>353.771111693891</v>
+        <v>352.2130440335152</v>
       </c>
     </row>
     <row r="6">
@@ -609,25 +609,25 @@
         <v>950</v>
       </c>
       <c r="C6" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D6" t="n">
-        <v>50.734619140625</v>
+        <v>-667.4052734375</v>
       </c>
       <c r="E6" t="n">
-        <v>7546.09375</v>
+        <v>7521.96826171875</v>
       </c>
       <c r="F6" t="n">
-        <v>56986195687.36523</v>
+        <v>56323154445.05591</v>
       </c>
       <c r="G6" t="n">
-        <v>5683.601787732804</v>
+        <v>5686.648527865045</v>
       </c>
       <c r="H6" t="n">
-        <v>118571.0881351793</v>
+        <v>117567.3584005246</v>
       </c>
       <c r="I6" t="n">
-        <v>344.3415283336869</v>
+        <v>342.8809682681799</v>
       </c>
     </row>
     <row r="7">
@@ -640,25 +640,25 @@
         <v>925</v>
       </c>
       <c r="C7" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D7" t="n">
-        <v>2381.0029296875</v>
+        <v>1636.52734375</v>
       </c>
       <c r="E7" t="n">
-        <v>9699.1630859375</v>
+        <v>9677.3974609375</v>
       </c>
       <c r="F7" t="n">
-        <v>79689262969.65063</v>
+        <v>78749802870.93628</v>
       </c>
       <c r="G7" t="n">
-        <v>7947.925493433777</v>
+        <v>7950.94761609158</v>
       </c>
       <c r="H7" t="n">
-        <v>112540.3054415104</v>
+        <v>111676.4764480491</v>
       </c>
       <c r="I7" t="n">
-        <v>335.4702750490875</v>
+        <v>334.1803052964808</v>
       </c>
     </row>
     <row r="8">
@@ -671,25 +671,25 @@
         <v>900</v>
       </c>
       <c r="C8" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D8" t="n">
-        <v>4762.21826171875</v>
+        <v>4009.0361328125</v>
       </c>
       <c r="E8" t="n">
-        <v>11911.2939453125</v>
+        <v>11898.005859375</v>
       </c>
       <c r="F8" t="n">
-        <v>102910447713.0308</v>
+        <v>101687648110.1216</v>
       </c>
       <c r="G8" t="n">
-        <v>10263.92440385074</v>
+        <v>10266.85952029883</v>
       </c>
       <c r="H8" t="n">
-        <v>107619.6883903062</v>
+        <v>106929.1387918027</v>
       </c>
       <c r="I8" t="n">
-        <v>328.0543985230287</v>
+        <v>327.000212219813</v>
       </c>
     </row>
     <row r="9">
@@ -702,25 +702,25 @@
         <v>875</v>
       </c>
       <c r="C9" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D9" t="n">
-        <v>7199.91796875</v>
+        <v>6452.4140625</v>
       </c>
       <c r="E9" t="n">
-        <v>14205.31640625</v>
+        <v>14181.26171875</v>
       </c>
       <c r="F9" t="n">
-        <v>126682940276.2607</v>
+        <v>125170208066.3564</v>
       </c>
       <c r="G9" t="n">
-        <v>12634.90880808245</v>
+        <v>12637.76836447405</v>
       </c>
       <c r="H9" t="n">
-        <v>104140.4987560865</v>
+        <v>103684.3255511515</v>
       </c>
       <c r="I9" t="n">
-        <v>322.7080704848989</v>
+        <v>322.0005055138136</v>
       </c>
     </row>
     <row r="10">
@@ -733,25 +733,25 @@
         <v>850</v>
       </c>
       <c r="C10" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D10" t="n">
-        <v>9703.72265625</v>
+        <v>8969.5859375</v>
       </c>
       <c r="E10" t="n">
-        <v>16554.390625</v>
+        <v>16519.91796875</v>
       </c>
       <c r="F10" t="n">
-        <v>151039716702.8516</v>
+        <v>149230516180.3008</v>
       </c>
       <c r="G10" t="n">
-        <v>15064.16762018232</v>
+        <v>15067.00935895018</v>
       </c>
       <c r="H10" t="n">
-        <v>102285.027405662</v>
+        <v>102149.0819664164</v>
       </c>
       <c r="I10" t="n">
-        <v>319.8203048676897</v>
+        <v>319.6077001050138</v>
       </c>
     </row>
     <row r="11">
@@ -764,25 +764,25 @@
         <v>825</v>
       </c>
       <c r="C11" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D11" t="n">
-        <v>12279.2109375</v>
+        <v>11560.8359375</v>
       </c>
       <c r="E11" t="n">
-        <v>18961.08203125</v>
+        <v>18918.2578125</v>
       </c>
       <c r="F11" t="n">
-        <v>176012794504.0391</v>
+        <v>173900176066.1172</v>
       </c>
       <c r="G11" t="n">
-        <v>17554.8941535819</v>
+        <v>17557.77335210444</v>
       </c>
       <c r="H11" t="n">
-        <v>101978.000511229</v>
+        <v>102250.6331069149</v>
       </c>
       <c r="I11" t="n">
-        <v>319.3399450604778</v>
+        <v>319.7665290597421</v>
       </c>
     </row>
     <row r="12">
@@ -795,25 +795,25 @@
         <v>800</v>
       </c>
       <c r="C12" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D12" t="n">
-        <v>14931.76171875</v>
+        <v>14227.22265625</v>
       </c>
       <c r="E12" t="n">
-        <v>21428.171875</v>
+        <v>21444.80078125</v>
       </c>
       <c r="F12" t="n">
-        <v>201632890778.4531</v>
+        <v>199209313744.3711</v>
       </c>
       <c r="G12" t="n">
-        <v>20110.1520231545</v>
+        <v>20113.10200756849</v>
       </c>
       <c r="H12" t="n">
-        <v>103094.8214974809</v>
+        <v>103851.1754513517</v>
       </c>
       <c r="I12" t="n">
-        <v>321.0838231637977</v>
+        <v>322.2594846569324</v>
       </c>
     </row>
     <row r="13">
@@ -826,25 +826,25 @@
         <v>775</v>
       </c>
       <c r="C13" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D13" t="n">
-        <v>17671.6328125</v>
+        <v>16971.20703125</v>
       </c>
       <c r="E13" t="n">
-        <v>24017.8671875</v>
+        <v>24061.49609375</v>
       </c>
       <c r="F13" t="n">
-        <v>227932347971.168</v>
+        <v>225189781031.6055</v>
       </c>
       <c r="G13" t="n">
-        <v>22733.16695008448</v>
+        <v>22736.21123338989</v>
       </c>
       <c r="H13" t="n">
-        <v>105363.2186831624</v>
+        <v>106679.7179003661</v>
       </c>
       <c r="I13" t="n">
-        <v>324.5970096645415</v>
+        <v>326.6186122993699</v>
       </c>
     </row>
     <row r="14">
@@ -857,25 +857,25 @@
         <v>750</v>
       </c>
       <c r="C14" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D14" t="n">
-        <v>20502.62890625</v>
+        <v>19797.12890625</v>
       </c>
       <c r="E14" t="n">
-        <v>26709.1796875</v>
+        <v>26747.9296875</v>
       </c>
       <c r="F14" t="n">
-        <v>254948868587.6484</v>
+        <v>251878898091.3867</v>
       </c>
       <c r="G14" t="n">
-        <v>25427.69924903916</v>
+        <v>25430.86904745248</v>
       </c>
       <c r="H14" t="n">
-        <v>108630.7976827274</v>
+        <v>110585.1471466864</v>
       </c>
       <c r="I14" t="n">
-        <v>329.5918653163749</v>
+        <v>332.5434515167701</v>
       </c>
     </row>
     <row r="15">
@@ -888,25 +888,25 @@
         <v>725</v>
       </c>
       <c r="C15" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D15" t="n">
-        <v>26421.2265625</v>
+        <v>25710.22265625</v>
       </c>
       <c r="E15" t="n">
         <v>32365.8828125</v>
       </c>
       <c r="F15" t="n">
-        <v>311301878224.5312</v>
+        <v>307549809113.6016</v>
       </c>
       <c r="G15" t="n">
-        <v>31048.14929756414</v>
+        <v>31051.66403538624</v>
       </c>
       <c r="H15" t="n">
-        <v>117349.6627435521</v>
+        <v>120749.3029137534</v>
       </c>
       <c r="I15" t="n">
-        <v>342.5633704054654</v>
+        <v>347.4900040486826</v>
       </c>
     </row>
     <row r="16">
@@ -919,25 +919,25 @@
         <v>700</v>
       </c>
       <c r="C16" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D16" t="n">
-        <v>31926.1953125</v>
+        <v>31469.72265625</v>
       </c>
       <c r="E16" t="n">
         <v>38350.328125</v>
       </c>
       <c r="F16" t="n">
-        <v>371069337126.7852</v>
+        <v>366593897988.8125</v>
       </c>
       <c r="G16" t="n">
-        <v>37009.14445029756</v>
+        <v>37013.0308016758</v>
       </c>
       <c r="H16" t="n">
-        <v>128424.704750733</v>
+        <v>133374.725734805</v>
       </c>
       <c r="I16" t="n">
-        <v>358.3639278034732</v>
+        <v>365.2050461518913</v>
       </c>
     </row>
     <row r="17">
@@ -950,25 +950,25 @@
         <v>650</v>
       </c>
       <c r="C17" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D17" t="n">
-        <v>37639.1796875</v>
+        <v>37117.0859375</v>
       </c>
       <c r="E17" t="n">
         <v>44689.9921875</v>
       </c>
       <c r="F17" t="n">
-        <v>434745270714.0078</v>
+        <v>429497314583.6523</v>
       </c>
       <c r="G17" t="n">
-        <v>43359.95705686945</v>
+        <v>43364.05330567436</v>
       </c>
       <c r="H17" t="n">
-        <v>142390.2501690685</v>
+        <v>148908.0236428283</v>
       </c>
       <c r="I17" t="n">
-        <v>377.3463265609836</v>
+        <v>385.8860241610576</v>
       </c>
     </row>
     <row r="18">
@@ -981,25 +981,25 @@
         <v>600</v>
       </c>
       <c r="C18" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D18" t="n">
-        <v>43742.5234375</v>
+        <v>43194.83203125</v>
       </c>
       <c r="E18" t="n">
-        <v>51450.26171875</v>
+        <v>51453.01171875</v>
       </c>
       <c r="F18" t="n">
-        <v>503014445019.2148</v>
+        <v>496935239204</v>
       </c>
       <c r="G18" t="n">
-        <v>50168.88326167911</v>
+        <v>50172.9009020689</v>
       </c>
       <c r="H18" t="n">
-        <v>161298.3398765762</v>
+        <v>169492.1050305835</v>
       </c>
       <c r="I18" t="n">
-        <v>401.6196457801539</v>
+        <v>411.6941887257864</v>
       </c>
     </row>
     <row r="19">
@@ -1012,25 +1012,25 @@
         <v>550</v>
       </c>
       <c r="C19" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D19" t="n">
-        <v>50245.98046875</v>
+        <v>49794.546875</v>
       </c>
       <c r="E19" t="n">
-        <v>58780.80859375</v>
+        <v>58785.05859375</v>
       </c>
       <c r="F19" t="n">
-        <v>576675784358.5039</v>
+        <v>569698475965.9414</v>
       </c>
       <c r="G19" t="n">
-        <v>57515.60495288333</v>
+        <v>57519.41686503104</v>
       </c>
       <c r="H19" t="n">
-        <v>189168.9907577027</v>
+        <v>199384.3246899957</v>
       </c>
       <c r="I19" t="n">
-        <v>434.9356167959836</v>
+        <v>446.5247190133999</v>
       </c>
     </row>
     <row r="20">
@@ -1043,25 +1043,25 @@
         <v>500</v>
       </c>
       <c r="C20" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D20" t="n">
-        <v>57320.828125</v>
+        <v>56983.375</v>
       </c>
       <c r="E20" t="n">
-        <v>66800.484375</v>
+        <v>66756.84375</v>
       </c>
       <c r="F20" t="n">
-        <v>656691741613.0039</v>
+        <v>648738657477.2188</v>
       </c>
       <c r="G20" t="n">
-        <v>65496.1137798598</v>
+        <v>65499.68246382237</v>
       </c>
       <c r="H20" t="n">
-        <v>231301.7860214092</v>
+        <v>244193.607674709</v>
       </c>
       <c r="I20" t="n">
-        <v>480.9384430687666</v>
+        <v>494.1594961899539</v>
       </c>
     </row>
     <row r="21">
@@ -1074,25 +1074,25 @@
         <v>450</v>
       </c>
       <c r="C21" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D21" t="n">
-        <v>65214.02734375</v>
+        <v>64909.421875</v>
       </c>
       <c r="E21" t="n">
-        <v>75588.890625</v>
+        <v>75491.3515625</v>
       </c>
       <c r="F21" t="n">
-        <v>744277001351.5781</v>
+        <v>735253276934.9453</v>
       </c>
       <c r="G21" t="n">
-        <v>74231.55808921905</v>
+        <v>74234.60220021645</v>
       </c>
       <c r="H21" t="n">
-        <v>294324.2188584534</v>
+        <v>310793.5513581467</v>
       </c>
       <c r="I21" t="n">
-        <v>542.5165609070874</v>
+        <v>557.4886109672077</v>
       </c>
     </row>
     <row r="22">
@@ -1105,25 +1105,25 @@
         <v>400</v>
       </c>
       <c r="C22" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D22" t="n">
-        <v>74065</v>
+        <v>73570</v>
       </c>
       <c r="E22" t="n">
-        <v>85314.6875</v>
+        <v>85183.5625</v>
       </c>
       <c r="F22" t="n">
-        <v>841055358257.5859</v>
+        <v>830846485381.6719</v>
       </c>
       <c r="G22" t="n">
-        <v>83883.88942473142</v>
+        <v>83886.13864989745</v>
       </c>
       <c r="H22" t="n">
-        <v>386642.5306040271</v>
+        <v>407808.8253914824</v>
       </c>
       <c r="I22" t="n">
-        <v>621.8058624715813</v>
+        <v>638.5991116431986</v>
       </c>
     </row>
     <row r="23">
@@ -1136,25 +1136,25 @@
         <v>350</v>
       </c>
       <c r="C23" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D23" t="n">
-        <v>83836.4375</v>
+        <v>83467.6875</v>
       </c>
       <c r="E23" t="n">
-        <v>96179.8125</v>
+        <v>96108.6875</v>
       </c>
       <c r="F23" t="n">
-        <v>949323544593</v>
+        <v>937788418727.625</v>
       </c>
       <c r="G23" t="n">
-        <v>94682.17574632539</v>
+        <v>94683.49532888229</v>
       </c>
       <c r="H23" t="n">
-        <v>516897.0087338662</v>
+        <v>543792.2484778526</v>
       </c>
       <c r="I23" t="n">
-        <v>718.9554984377448</v>
+        <v>737.4227067821091</v>
       </c>
     </row>
     <row r="24">
@@ -1167,25 +1167,25 @@
         <v>300</v>
       </c>
       <c r="C24" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D24" t="n">
-        <v>95370.125</v>
+        <v>95173.625</v>
       </c>
       <c r="E24" t="n">
         <v>108594.3125</v>
       </c>
       <c r="F24" t="n">
-        <v>1072548696688.875</v>
+        <v>1059507117999.188</v>
       </c>
       <c r="G24" t="n">
-        <v>106972.2169799613</v>
+        <v>106972.7832575529</v>
       </c>
       <c r="H24" t="n">
-        <v>686421.3064129201</v>
+        <v>718045.5007289799</v>
       </c>
       <c r="I24" t="n">
-        <v>828.5054655299023</v>
+        <v>847.37565502496</v>
       </c>
     </row>
     <row r="25">
@@ -1198,25 +1198,25 @@
         <v>250</v>
       </c>
       <c r="C25" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D25" t="n">
-        <v>102082.0625</v>
+        <v>101950.5625</v>
       </c>
       <c r="E25" t="n">
         <v>115556.1875</v>
       </c>
       <c r="F25" t="n">
-        <v>1141391854346</v>
+        <v>1127511967707.625</v>
       </c>
       <c r="G25" t="n">
-        <v>113838.390256026</v>
+        <v>113838.8702566292</v>
       </c>
       <c r="H25" t="n">
-        <v>775708.1545666415</v>
+        <v>807606.2457732505</v>
       </c>
       <c r="I25" t="n">
-        <v>880.7429560130705</v>
+        <v>898.669152565754</v>
       </c>
     </row>
     <row r="26">
@@ -1229,25 +1229,25 @@
         <v>200</v>
       </c>
       <c r="C26" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D26" t="n">
-        <v>109609.875</v>
+        <v>109531.375</v>
       </c>
       <c r="E26" t="n">
         <v>123144.6875</v>
       </c>
       <c r="F26" t="n">
-        <v>1216395987873.125</v>
+        <v>1201605377631.812</v>
       </c>
       <c r="G26" t="n">
-        <v>121319.0374945407</v>
+        <v>121319.6867098505</v>
       </c>
       <c r="H26" t="n">
-        <v>846740.6260925599</v>
+        <v>876553.8941034599</v>
       </c>
       <c r="I26" t="n">
-        <v>920.1851042548776</v>
+        <v>936.2445695989162</v>
       </c>
     </row>
     <row r="27">
@@ -1260,25 +1260,25 @@
         <v>150</v>
       </c>
       <c r="C27" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D27" t="n">
-        <v>118110.75</v>
+        <v>118047.75</v>
       </c>
       <c r="E27" t="n">
         <v>131516.5625</v>
       </c>
       <c r="F27" t="n">
-        <v>1299099068600.562</v>
+        <v>1283308347025.375</v>
       </c>
       <c r="G27" t="n">
-        <v>129567.5505213141</v>
+        <v>129568.7998002286</v>
       </c>
       <c r="H27" t="n">
-        <v>865795.0590049953</v>
+        <v>891515.1865617182</v>
       </c>
       <c r="I27" t="n">
-        <v>930.4810900845838</v>
+        <v>944.2008189795846</v>
       </c>
     </row>
     <row r="28">
@@ -1291,25 +1291,25 @@
         <v>100</v>
       </c>
       <c r="C28" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D28" t="n">
-        <v>127869.875</v>
+        <v>127832.875</v>
       </c>
       <c r="E28" t="n">
-        <v>140866.1875</v>
+        <v>140910.1875</v>
       </c>
       <c r="F28" t="n">
-        <v>1391879173863.688</v>
+        <v>1374969015143.625</v>
       </c>
       <c r="G28" t="n">
-        <v>138821.1103664469</v>
+        <v>138823.2886255346</v>
       </c>
       <c r="H28" t="n">
-        <v>791618.533078799</v>
+        <v>813139.4504046426</v>
       </c>
       <c r="I28" t="n">
-        <v>889.7294718501793</v>
+        <v>901.7424523691022</v>
       </c>
     </row>
     <row r="29">
@@ -1322,25 +1322,25 @@
         <v>1000</v>
       </c>
       <c r="C29" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D29" t="n">
-        <v>-2.138814926147461</v>
+        <v>-2.018579483032227</v>
       </c>
       <c r="E29" t="n">
-        <v>1.7308349609375</v>
+        <v>1.798852920532227</v>
       </c>
       <c r="F29" t="n">
-        <v>-2422.814295768738</v>
+        <v>-2545.117341995239</v>
       </c>
       <c r="G29" t="n">
-        <v>-0.0002416429364459035</v>
+        <v>-0.0002569669246813929</v>
       </c>
       <c r="H29" t="n">
-        <v>0.003718447210900799</v>
+        <v>0.003622592962962754</v>
       </c>
       <c r="I29" t="n">
-        <v>0.060979071909146</v>
+        <v>0.06018798021999704</v>
       </c>
     </row>
     <row r="30">
@@ -1353,25 +1353,25 @@
         <v>975</v>
       </c>
       <c r="C30" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D30" t="n">
-        <v>-2.400935173034668</v>
+        <v>-2.665791511535645</v>
       </c>
       <c r="E30" t="n">
-        <v>2.099066734313965</v>
+        <v>2.307659149169922</v>
       </c>
       <c r="F30" t="n">
-        <v>-11428.87547302246</v>
+        <v>-10187.47474384308</v>
       </c>
       <c r="G30" t="n">
-        <v>-0.001139875653862042</v>
+        <v>-0.001028574994166067</v>
       </c>
       <c r="H30" t="n">
-        <v>0.008556248384394498</v>
+        <v>0.008391431594142275</v>
       </c>
       <c r="I30" t="n">
-        <v>0.09249999126699687</v>
+        <v>0.09160475748640065</v>
       </c>
     </row>
     <row r="31">
@@ -1384,25 +1384,25 @@
         <v>950</v>
       </c>
       <c r="C31" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D31" t="n">
-        <v>-4.727029800415039</v>
+        <v>-4.483035087585449</v>
       </c>
       <c r="E31" t="n">
         <v>2.412403106689453</v>
       </c>
       <c r="F31" t="n">
-        <v>-23667.27976608276</v>
+        <v>-21250.07687282562</v>
       </c>
       <c r="G31" t="n">
-        <v>-0.002360490851631011</v>
+        <v>-0.002145506933276555</v>
       </c>
       <c r="H31" t="n">
-        <v>0.01652364976495156</v>
+        <v>0.01629225734534536</v>
       </c>
       <c r="I31" t="n">
-        <v>0.1285443494088774</v>
+        <v>0.1276411271704593</v>
       </c>
     </row>
     <row r="32">
@@ -1415,25 +1415,25 @@
         <v>925</v>
       </c>
       <c r="C32" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D32" t="n">
-        <v>-6.604527473449707</v>
+        <v>-6.002691268920898</v>
       </c>
       <c r="E32" t="n">
-        <v>2.899991035461426</v>
+        <v>2.613036155700684</v>
       </c>
       <c r="F32" t="n">
-        <v>-34448.7924823761</v>
+        <v>-30916.20142173767</v>
       </c>
       <c r="G32" t="n">
-        <v>-0.003435800831699997</v>
+        <v>-0.003121443978667936</v>
       </c>
       <c r="H32" t="n">
-        <v>0.02449627987137436</v>
+        <v>0.02425014423273291</v>
       </c>
       <c r="I32" t="n">
-        <v>0.1565128744588584</v>
+        <v>0.1557245781266814</v>
       </c>
     </row>
     <row r="33">
@@ -1446,25 +1446,25 @@
         <v>900</v>
       </c>
       <c r="C33" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D33" t="n">
-        <v>-7.907404899597168</v>
+        <v>-7.213781356811523</v>
       </c>
       <c r="E33" t="n">
-        <v>3.30113410949707</v>
+        <v>3.39769172668457</v>
       </c>
       <c r="F33" t="n">
-        <v>-42482.3123884201</v>
+        <v>-37831.50194644928</v>
       </c>
       <c r="G33" t="n">
-        <v>-0.004237035719360724</v>
+        <v>-0.003819644992727925</v>
       </c>
       <c r="H33" t="n">
-        <v>0.03083903847651879</v>
+        <v>0.03058255758319868</v>
       </c>
       <c r="I33" t="n">
-        <v>0.1756104737096247</v>
+        <v>0.1748786939086597</v>
       </c>
     </row>
     <row r="34">
@@ -1477,25 +1477,25 @@
         <v>875</v>
       </c>
       <c r="C34" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D34" t="n">
-        <v>-8.800127029418945</v>
+        <v>-8.089030265808105</v>
       </c>
       <c r="E34" t="n">
-        <v>3.340728759765625</v>
+        <v>4.389358520507812</v>
       </c>
       <c r="F34" t="n">
-        <v>-47918.9500875473</v>
+        <v>-42149.72807216644</v>
       </c>
       <c r="G34" t="n">
-        <v>-0.004779266752215353</v>
+        <v>-0.004255633255153008</v>
       </c>
       <c r="H34" t="n">
-        <v>0.03531862348755055</v>
+        <v>0.03500458133462445</v>
       </c>
       <c r="I34" t="n">
-        <v>0.1879324971566933</v>
+        <v>0.187095113069862</v>
       </c>
     </row>
     <row r="35">
@@ -1508,25 +1508,25 @@
         <v>850</v>
       </c>
       <c r="C35" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D35" t="n">
-        <v>-9.277047157287598</v>
+        <v>-9.663198471069336</v>
       </c>
       <c r="E35" t="n">
-        <v>3.411510467529297</v>
+        <v>5.186410903930664</v>
       </c>
       <c r="F35" t="n">
-        <v>-51821.69149208069</v>
+        <v>-44967.81840610504</v>
       </c>
       <c r="G35" t="n">
-        <v>-0.005168512388922798</v>
+        <v>-0.004540160807041402</v>
       </c>
       <c r="H35" t="n">
-        <v>0.03841090067414073</v>
+        <v>0.03799295427840122</v>
       </c>
       <c r="I35" t="n">
-        <v>0.1959869910839511</v>
+        <v>0.1949178141638194</v>
       </c>
     </row>
     <row r="36">
@@ -1539,25 +1539,25 @@
         <v>825</v>
       </c>
       <c r="C36" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D36" t="n">
-        <v>-11.21321201324463</v>
+        <v>-10.84944725036621</v>
       </c>
       <c r="E36" t="n">
-        <v>3.772537231445312</v>
+        <v>5.845376968383789</v>
       </c>
       <c r="F36" t="n">
-        <v>-55127.48630332947</v>
+        <v>-47130.8146314621</v>
       </c>
       <c r="G36" t="n">
-        <v>-0.00549822068182539</v>
+        <v>-0.004758547000462133</v>
       </c>
       <c r="H36" t="n">
-        <v>0.04066114822639713</v>
+        <v>0.04013955172505033</v>
       </c>
       <c r="I36" t="n">
-        <v>0.2016460964819233</v>
+        <v>0.2003485755503401</v>
       </c>
     </row>
     <row r="37">
@@ -1570,25 +1570,25 @@
         <v>800</v>
       </c>
       <c r="C37" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D37" t="n">
-        <v>-12.87025260925293</v>
+        <v>-11.63267517089844</v>
       </c>
       <c r="E37" t="n">
-        <v>4.08746337890625</v>
+        <v>6.301895141601562</v>
       </c>
       <c r="F37" t="n">
-        <v>-57937.18080806732</v>
+        <v>-48777.04995441437</v>
       </c>
       <c r="G37" t="n">
-        <v>-0.005778449683208786</v>
+        <v>-0.004924758601499451</v>
       </c>
       <c r="H37" t="n">
-        <v>0.04220286075598235</v>
+        <v>0.0416425576762125</v>
       </c>
       <c r="I37" t="n">
-        <v>0.2054333486948562</v>
+        <v>0.2040650819621341</v>
       </c>
     </row>
     <row r="38">
@@ -1601,25 +1601,25 @@
         <v>775</v>
       </c>
       <c r="C38" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D38" t="n">
-        <v>-13.91684150695801</v>
+        <v>-12.10081577301025</v>
       </c>
       <c r="E38" t="n">
-        <v>4.463313102722168</v>
+        <v>6.637953758239746</v>
       </c>
       <c r="F38" t="n">
-        <v>-59398.15040111542</v>
+        <v>-49135.34728908539</v>
       </c>
       <c r="G38" t="n">
-        <v>-0.005924161627842294</v>
+        <v>-0.004960933972549249</v>
       </c>
       <c r="H38" t="n">
-        <v>0.04342311519861047</v>
+        <v>0.04284451436138358</v>
       </c>
       <c r="I38" t="n">
-        <v>0.2083821374269169</v>
+        <v>0.2069891648405384</v>
       </c>
     </row>
     <row r="39">
@@ -1632,25 +1632,25 @@
         <v>750</v>
       </c>
       <c r="C39" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D39" t="n">
-        <v>-14.50279140472412</v>
+        <v>-12.29857349395752</v>
       </c>
       <c r="E39" t="n">
-        <v>4.735078811645508</v>
+        <v>6.95191478729248</v>
       </c>
       <c r="F39" t="n">
-        <v>-60723.82324504852</v>
+        <v>-49356.79205036163</v>
       </c>
       <c r="G39" t="n">
-        <v>-0.006056379552812455</v>
+        <v>-0.004983292069110488</v>
       </c>
       <c r="H39" t="n">
-        <v>0.04459916147186013</v>
+        <v>0.0439999258187638</v>
       </c>
       <c r="I39" t="n">
-        <v>0.2111851355371872</v>
+        <v>0.2097615928113719</v>
       </c>
     </row>
     <row r="40">
@@ -1663,25 +1663,25 @@
         <v>725</v>
       </c>
       <c r="C40" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D40" t="n">
-        <v>-14.14280891418457</v>
+        <v>-13.4630069732666</v>
       </c>
       <c r="E40" t="n">
-        <v>6.10694408416748</v>
+        <v>7.426641464233398</v>
       </c>
       <c r="F40" t="n">
-        <v>-62648.70530414581</v>
+        <v>-48921.56094264984</v>
       </c>
       <c r="G40" t="n">
-        <v>-0.006248360487498465</v>
+        <v>-0.004939349105291446</v>
       </c>
       <c r="H40" t="n">
-        <v>0.04701351997328641</v>
+        <v>0.04641202569741818</v>
       </c>
       <c r="I40" t="n">
-        <v>0.2168260131379222</v>
+        <v>0.2154345044263295</v>
       </c>
     </row>
     <row r="41">
@@ -1694,25 +1694,25 @@
         <v>700</v>
       </c>
       <c r="C41" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D41" t="n">
-        <v>-14.72065544128418</v>
+        <v>-14.41956996917725</v>
       </c>
       <c r="E41" t="n">
-        <v>5.051517486572266</v>
+        <v>7.039414405822754</v>
       </c>
       <c r="F41" t="n">
-        <v>-65569.61175251007</v>
+        <v>-49406.89451408386</v>
       </c>
       <c r="G41" t="n">
-        <v>-0.006539681375153486</v>
+        <v>-0.004988350647671554</v>
       </c>
       <c r="H41" t="n">
-        <v>0.04905054993134285</v>
+        <v>0.04848868350143795</v>
       </c>
       <c r="I41" t="n">
-        <v>0.2214735874350322</v>
+        <v>0.2202014611700793</v>
       </c>
     </row>
     <row r="42">
@@ -1725,25 +1725,25 @@
         <v>650</v>
       </c>
       <c r="C42" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D42" t="n">
-        <v>-15.0778169631958</v>
+        <v>-14.66117763519287</v>
       </c>
       <c r="E42" t="n">
-        <v>4.582921981811523</v>
+        <v>5.498002052307129</v>
       </c>
       <c r="F42" t="n">
-        <v>-67779.94095611572</v>
+        <v>-49743.17499542236</v>
       </c>
       <c r="G42" t="n">
-        <v>-0.006760131799358101</v>
+        <v>-0.005022303094458242</v>
       </c>
       <c r="H42" t="n">
-        <v>0.04832009215640842</v>
+        <v>0.04790965919091781</v>
       </c>
       <c r="I42" t="n">
-        <v>0.2198183162441393</v>
+        <v>0.218882752154933</v>
       </c>
     </row>
     <row r="43">
@@ -1756,25 +1756,25 @@
         <v>600</v>
       </c>
       <c r="C43" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D43" t="n">
-        <v>-14.58753776550293</v>
+        <v>-14.94180870056152</v>
       </c>
       <c r="E43" t="n">
-        <v>3.555633544921875</v>
+        <v>6.040891647338867</v>
       </c>
       <c r="F43" t="n">
-        <v>-70852.97952270508</v>
+        <v>-51427.74940872192</v>
       </c>
       <c r="G43" t="n">
-        <v>-0.007066625806900938</v>
+        <v>-0.005192385588982109</v>
       </c>
       <c r="H43" t="n">
-        <v>0.04741564897971055</v>
+        <v>0.04690278074480758</v>
       </c>
       <c r="I43" t="n">
-        <v>0.2177513466771458</v>
+        <v>0.2165704983251587</v>
       </c>
     </row>
     <row r="44">
@@ -1787,25 +1787,25 @@
         <v>550</v>
       </c>
       <c r="C44" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D44" t="n">
-        <v>-14.42328262329102</v>
+        <v>-15.25595188140869</v>
       </c>
       <c r="E44" t="n">
-        <v>2.957959175109863</v>
+        <v>6.178739547729492</v>
       </c>
       <c r="F44" t="n">
-        <v>-71383.06396961212</v>
+        <v>-51414.62700843811</v>
       </c>
       <c r="G44" t="n">
-        <v>-0.007119494556494621</v>
+        <v>-0.005191060690208411</v>
       </c>
       <c r="H44" t="n">
-        <v>0.04685177605657885</v>
+        <v>0.04604575138372741</v>
       </c>
       <c r="I44" t="n">
-        <v>0.2164527109014319</v>
+        <v>0.2145827378512247</v>
       </c>
     </row>
     <row r="45">
@@ -1818,25 +1818,25 @@
         <v>500</v>
       </c>
       <c r="C45" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D45" t="n">
-        <v>-14.67950439453125</v>
+        <v>-14.8433780670166</v>
       </c>
       <c r="E45" t="n">
-        <v>2.667131423950195</v>
+        <v>5.498003005981445</v>
       </c>
       <c r="F45" t="n">
-        <v>-72032.88622665405</v>
+        <v>-51868.24850749969</v>
       </c>
       <c r="G45" t="n">
-        <v>-0.007184305532157776</v>
+        <v>-0.005236860433764368</v>
       </c>
       <c r="H45" t="n">
-        <v>0.0460781127435935</v>
+        <v>0.04495171849315378</v>
       </c>
       <c r="I45" t="n">
-        <v>0.2146581299266196</v>
+        <v>0.2120182032117851</v>
       </c>
     </row>
     <row r="46">
@@ -1849,25 +1849,25 @@
         <v>450</v>
       </c>
       <c r="C46" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D46" t="n">
-        <v>-14.51239013671875</v>
+        <v>-14.42695903778076</v>
       </c>
       <c r="E46" t="n">
-        <v>2.369221687316895</v>
+        <v>3.790817260742188</v>
       </c>
       <c r="F46" t="n">
-        <v>-73099.54794216156</v>
+        <v>-52945.61805725098</v>
       </c>
       <c r="G46" t="n">
-        <v>-0.007290690602437312</v>
+        <v>-0.005345636691494003</v>
       </c>
       <c r="H46" t="n">
-        <v>0.04292757610627798</v>
+        <v>0.04164679652687933</v>
       </c>
       <c r="I46" t="n">
-        <v>0.207189710425682</v>
+        <v>0.2040754677242694</v>
       </c>
     </row>
     <row r="47">
@@ -1880,25 +1880,25 @@
         <v>400</v>
       </c>
       <c r="C47" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D47" t="n">
         <v>-13.51175689697266</v>
       </c>
       <c r="E47" t="n">
-        <v>1.987301826477051</v>
+        <v>2.974142074584961</v>
       </c>
       <c r="F47" t="n">
-        <v>-71394.13938236237</v>
+        <v>-52356.18314743042</v>
       </c>
       <c r="G47" t="n">
-        <v>-0.007120599179025518</v>
+        <v>-0.005286124592158797</v>
       </c>
       <c r="H47" t="n">
-        <v>0.03697289233558221</v>
+        <v>0.03573288526472417</v>
       </c>
       <c r="I47" t="n">
-        <v>0.1922833646875938</v>
+        <v>0.18903143988428</v>
       </c>
     </row>
     <row r="48">
@@ -1911,25 +1911,25 @@
         <v>350</v>
       </c>
       <c r="C48" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D48" t="n">
         <v>-11.9915885925293</v>
       </c>
       <c r="E48" t="n">
-        <v>1.664351463317871</v>
+        <v>2.847209930419922</v>
       </c>
       <c r="F48" t="n">
-        <v>-62053.81642627716</v>
+        <v>-45868.96747303009</v>
       </c>
       <c r="G48" t="n">
-        <v>-0.006189028372957861</v>
+        <v>-0.004631145022419724</v>
       </c>
       <c r="H48" t="n">
-        <v>0.02904300422453121</v>
+        <v>0.02806401425373653</v>
       </c>
       <c r="I48" t="n">
-        <v>0.1704200816351501</v>
+        <v>0.1675231752735619</v>
       </c>
     </row>
     <row r="49">
@@ -1942,25 +1942,25 @@
         <v>300</v>
       </c>
       <c r="C49" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D49" t="n">
-        <v>-9.580441474914551</v>
+        <v>-10.08780384063721</v>
       </c>
       <c r="E49" t="n">
-        <v>1.486281394958496</v>
+        <v>2.621424674987793</v>
       </c>
       <c r="F49" t="n">
-        <v>-43618.08973026276</v>
+        <v>-32174.1876077652</v>
       </c>
       <c r="G49" t="n">
-        <v>-0.004350314137979509</v>
+        <v>-0.003248456134917587</v>
       </c>
       <c r="H49" t="n">
-        <v>0.02057371278655632</v>
+        <v>0.0198978685735314</v>
       </c>
       <c r="I49" t="n">
-        <v>0.1434353958636303</v>
+        <v>0.1410598049535423</v>
       </c>
     </row>
     <row r="50">
@@ -1973,25 +1973,25 @@
         <v>250</v>
       </c>
       <c r="C50" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D50" t="n">
-        <v>-8.87787914276123</v>
+        <v>-9.601442337036133</v>
       </c>
       <c r="E50" t="n">
-        <v>1.505794525146484</v>
+        <v>2.766477584838867</v>
       </c>
       <c r="F50" t="n">
-        <v>-33490.62929344177</v>
+        <v>-24422.53395557404</v>
       </c>
       <c r="G50" t="n">
-        <v>-0.003340237021063417</v>
+        <v>-0.002465813005922479</v>
       </c>
       <c r="H50" t="n">
-        <v>0.0160246975916697</v>
+        <v>0.01550333379751017</v>
       </c>
       <c r="I50" t="n">
-        <v>0.1265886945649954</v>
+        <v>0.1245123841130278</v>
       </c>
     </row>
     <row r="51">
@@ -2004,25 +2004,25 @@
         <v>200</v>
       </c>
       <c r="C51" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D51" t="n">
-        <v>-7.655767440795898</v>
+        <v>-8.764391899108887</v>
       </c>
       <c r="E51" t="n">
-        <v>1.579972267150879</v>
+        <v>3.319348335266113</v>
       </c>
       <c r="F51" t="n">
-        <v>-24104.18044757843</v>
+        <v>-17577.10592746735</v>
       </c>
       <c r="G51" t="n">
-        <v>-0.002404065781742746</v>
+        <v>-0.001774666645208374</v>
       </c>
       <c r="H51" t="n">
-        <v>0.01105741416900901</v>
+        <v>0.01069777299772647</v>
       </c>
       <c r="I51" t="n">
-        <v>0.105154239900296</v>
+        <v>0.1034300391459197</v>
       </c>
     </row>
     <row r="52">
@@ -2035,25 +2035,25 @@
         <v>150</v>
       </c>
       <c r="C52" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D52" t="n">
-        <v>-5.896099090576172</v>
+        <v>-7.643311500549316</v>
       </c>
       <c r="E52" t="n">
-        <v>1.70118522644043</v>
+        <v>3.166014671325684</v>
       </c>
       <c r="F52" t="n">
-        <v>-15835.83107471466</v>
+        <v>-12195.98041915894</v>
       </c>
       <c r="G52" t="n">
-        <v>-0.001579409832870084</v>
+        <v>-0.001231363100661162</v>
       </c>
       <c r="H52" t="n">
-        <v>0.006414038617623939</v>
+        <v>0.006217648357252597</v>
       </c>
       <c r="I52" t="n">
-        <v>0.08008769329693508</v>
+        <v>0.07885206628397633</v>
       </c>
     </row>
     <row r="53">
@@ -2066,25 +2066,25 @@
         <v>100</v>
       </c>
       <c r="C53" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D53" t="n">
-        <v>-3.676130294799805</v>
+        <v>-6.201698303222656</v>
       </c>
       <c r="E53" t="n">
-        <v>1.266777038574219</v>
+        <v>2.209678649902344</v>
       </c>
       <c r="F53" t="n">
-        <v>-8666.518324315548</v>
+        <v>-7296.581416249275</v>
       </c>
       <c r="G53" t="n">
-        <v>-0.0008643679130947845</v>
+        <v>-0.0007366969122732421</v>
       </c>
       <c r="H53" t="n">
-        <v>0.003069765605709968</v>
+        <v>0.003006586844945881</v>
       </c>
       <c r="I53" t="n">
-        <v>0.05540546548590642</v>
+        <v>0.05483235217411233</v>
       </c>
     </row>
     <row r="54">
@@ -2097,25 +2097,25 @@
         <v>1000</v>
       </c>
       <c r="C54" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D54" t="n">
-        <v>5.437365531921387</v>
+        <v>5.067600250244141</v>
       </c>
       <c r="E54" t="n">
-        <v>108.203727722168</v>
+        <v>116.6183471679688</v>
       </c>
       <c r="F54" t="n">
-        <v>799480648.9655766</v>
+        <v>788589479.3050032</v>
       </c>
       <c r="G54" t="n">
-        <v>79.73737483104152</v>
+        <v>79.61967410675287</v>
       </c>
       <c r="H54" t="n">
-        <v>141.5479151988288</v>
+        <v>140.606027165696</v>
       </c>
       <c r="I54" t="n">
-        <v>11.89739110892925</v>
+        <v>11.85774123371294</v>
       </c>
     </row>
     <row r="55">
@@ -2128,25 +2128,25 @@
         <v>975</v>
       </c>
       <c r="C55" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D55" t="n">
-        <v>4.126392364501953</v>
+        <v>5.196361541748047</v>
       </c>
       <c r="E55" t="n">
-        <v>108.0694427490234</v>
+        <v>116.6277618408203</v>
       </c>
       <c r="F55" t="n">
-        <v>845822823.3023</v>
+        <v>835021803.2158451</v>
       </c>
       <c r="G55" t="n">
-        <v>84.35937954166702</v>
+        <v>84.30769822426825</v>
       </c>
       <c r="H55" t="n">
-        <v>165.8345788801995</v>
+        <v>163.5782981486893</v>
       </c>
       <c r="I55" t="n">
-        <v>12.87767754217349</v>
+        <v>12.78977318597516</v>
       </c>
     </row>
     <row r="56">
@@ -2159,25 +2159,25 @@
         <v>950</v>
       </c>
       <c r="C56" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D56" t="n">
-        <v>0.02105144038796425</v>
+        <v>1.62249755859375</v>
       </c>
       <c r="E56" t="n">
-        <v>108.5846328735352</v>
+        <v>117.5825347900391</v>
       </c>
       <c r="F56" t="n">
-        <v>846053103.6325303</v>
+        <v>835802388.3034761</v>
       </c>
       <c r="G56" t="n">
-        <v>84.38234688807047</v>
+        <v>84.38650973763586</v>
       </c>
       <c r="H56" t="n">
-        <v>184.7366466254045</v>
+        <v>179.4135952790548</v>
       </c>
       <c r="I56" t="n">
-        <v>13.59178599836697</v>
+        <v>13.39453602328408</v>
       </c>
     </row>
     <row r="57">
@@ -2190,25 +2190,25 @@
         <v>925</v>
       </c>
       <c r="C57" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D57" t="n">
-        <v>0.4477879405021667</v>
+        <v>0.09112149477005005</v>
       </c>
       <c r="E57" t="n">
-        <v>109.2074737548828</v>
+        <v>117.4900207519531</v>
       </c>
       <c r="F57" t="n">
-        <v>806131517.6582989</v>
+        <v>797110613.5747745</v>
       </c>
       <c r="G57" t="n">
-        <v>80.40070897251194</v>
+        <v>80.48000758999579</v>
       </c>
       <c r="H57" t="n">
-        <v>211.5394880794512</v>
+        <v>204.369187329616</v>
       </c>
       <c r="I57" t="n">
-        <v>14.54439713702329</v>
+        <v>14.29577515665436</v>
       </c>
     </row>
     <row r="58">
@@ -2221,25 +2221,25 @@
         <v>900</v>
       </c>
       <c r="C58" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D58" t="n">
-        <v>-0.9287099838256836</v>
+        <v>-0.2024116516113281</v>
       </c>
       <c r="E58" t="n">
-        <v>110.0415496826172</v>
+        <v>117.3299407958984</v>
       </c>
       <c r="F58" t="n">
-        <v>767206354.0854805</v>
+        <v>758518382.7094388</v>
       </c>
       <c r="G58" t="n">
-        <v>76.5184507062467</v>
+        <v>76.58355585536411</v>
       </c>
       <c r="H58" t="n">
-        <v>262.6125286123836</v>
+        <v>256.7416559077095</v>
       </c>
       <c r="I58" t="n">
-        <v>16.20532408230035</v>
+        <v>16.02315998508751</v>
       </c>
     </row>
     <row r="59">
@@ -2252,25 +2252,25 @@
         <v>875</v>
       </c>
       <c r="C59" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D59" t="n">
         <v>-0.9581308364868164</v>
       </c>
       <c r="E59" t="n">
-        <v>110.1420669555664</v>
+        <v>114.7705993652344</v>
       </c>
       <c r="F59" t="n">
-        <v>726642248.4071285</v>
+        <v>717247450.6439204</v>
       </c>
       <c r="G59" t="n">
-        <v>72.47273014584832</v>
+        <v>72.41664994630355</v>
       </c>
       <c r="H59" t="n">
-        <v>336.8494977824636</v>
+        <v>336.570999226416</v>
       </c>
       <c r="I59" t="n">
-        <v>18.35346010381867</v>
+        <v>18.34587144908674</v>
       </c>
     </row>
     <row r="60">
@@ -2283,25 +2283,25 @@
         <v>850</v>
       </c>
       <c r="C60" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D60" t="n">
         <v>-3.572824478149414</v>
       </c>
       <c r="E60" t="n">
-        <v>122.3688888549805</v>
+        <v>115.5573806762695</v>
       </c>
       <c r="F60" t="n">
-        <v>684961951.1587551</v>
+        <v>675139288.3842309</v>
       </c>
       <c r="G60" t="n">
-        <v>68.31568458250334</v>
+        <v>68.16521336956298</v>
       </c>
       <c r="H60" t="n">
-        <v>416.3709013661519</v>
+        <v>419.277882977458</v>
       </c>
       <c r="I60" t="n">
-        <v>20.40516849639208</v>
+        <v>20.47627610131925</v>
       </c>
     </row>
     <row r="61">
@@ -2314,25 +2314,25 @@
         <v>825</v>
       </c>
       <c r="C61" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D61" t="n">
-        <v>-4.339694976806641</v>
+        <v>-5.618928909301758</v>
       </c>
       <c r="E61" t="n">
-        <v>115.7575988769531</v>
+        <v>116.4183731079102</v>
       </c>
       <c r="F61" t="n">
-        <v>646965462.1959532</v>
+        <v>637129889.2165781</v>
       </c>
       <c r="G61" t="n">
-        <v>64.52604904021635</v>
+        <v>64.3276070431514</v>
       </c>
       <c r="H61" t="n">
-        <v>476.3767486871807</v>
+        <v>479.7062667121182</v>
       </c>
       <c r="I61" t="n">
-        <v>21.82605664537643</v>
+        <v>21.90219775986233</v>
       </c>
     </row>
     <row r="62">
@@ -2345,25 +2345,25 @@
         <v>800</v>
       </c>
       <c r="C62" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D62" t="n">
-        <v>-5.542159080505371</v>
+        <v>-3.283346176147461</v>
       </c>
       <c r="E62" t="n">
-        <v>115.3020858764648</v>
+        <v>116.4541397094727</v>
       </c>
       <c r="F62" t="n">
-        <v>614790993.5980947</v>
+        <v>605409706.1707394</v>
       </c>
       <c r="G62" t="n">
-        <v>61.31708123605928</v>
+        <v>61.12498932760446</v>
       </c>
       <c r="H62" t="n">
-        <v>513.1041442007436</v>
+        <v>514.3013910427478</v>
       </c>
       <c r="I62" t="n">
-        <v>22.65180222853677</v>
+        <v>22.67821401792363</v>
       </c>
     </row>
     <row r="63">
@@ -2376,25 +2376,25 @@
         <v>775</v>
       </c>
       <c r="C63" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D63" t="n">
-        <v>-3.032523155212402</v>
+        <v>-5.978819847106934</v>
       </c>
       <c r="E63" t="n">
-        <v>112.8669815063477</v>
+        <v>120.837776184082</v>
       </c>
       <c r="F63" t="n">
-        <v>586976379.7173281</v>
+        <v>577915154.0804738</v>
       </c>
       <c r="G63" t="n">
-        <v>58.54294993511908</v>
+        <v>58.34901103397174</v>
       </c>
       <c r="H63" t="n">
-        <v>536.4232597026821</v>
+        <v>535.9126250883144</v>
       </c>
       <c r="I63" t="n">
-        <v>23.16081301903459</v>
+        <v>23.14978671798758</v>
       </c>
     </row>
     <row r="64">
@@ -2407,25 +2407,25 @@
         <v>750</v>
       </c>
       <c r="C64" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D64" t="n">
-        <v>-5.241782188415527</v>
+        <v>-5.913242340087891</v>
       </c>
       <c r="E64" t="n">
-        <v>114.5705184936523</v>
+        <v>115.3855743408203</v>
       </c>
       <c r="F64" t="n">
-        <v>561572819.367018</v>
+        <v>552534237.0440724</v>
       </c>
       <c r="G64" t="n">
-        <v>56.00928859345133</v>
+        <v>55.78643519952108</v>
       </c>
       <c r="H64" t="n">
-        <v>545.0898531239231</v>
+        <v>543.2771864136471</v>
       </c>
       <c r="I64" t="n">
-        <v>23.34715942302025</v>
+        <v>23.30830724041639</v>
       </c>
     </row>
     <row r="65">
@@ -2438,25 +2438,25 @@
         <v>725</v>
       </c>
       <c r="C65" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D65" t="n">
         <v>-6.19677734375</v>
       </c>
       <c r="E65" t="n">
-        <v>114.904670715332</v>
+        <v>112.7630233764648</v>
       </c>
       <c r="F65" t="n">
-        <v>519284117.4072941</v>
+        <v>509840291.6445113</v>
       </c>
       <c r="G65" t="n">
-        <v>51.7915628940942</v>
+        <v>51.47585522318095</v>
       </c>
       <c r="H65" t="n">
-        <v>545.8643188104913</v>
+        <v>540.5429482536663</v>
       </c>
       <c r="I65" t="n">
-        <v>23.36373940127075</v>
+        <v>23.24957952853484</v>
       </c>
     </row>
     <row r="66">
@@ -2469,7 +2469,7 @@
         <v>700</v>
       </c>
       <c r="C66" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D66" t="n">
         <v>-9.847058296203613</v>
@@ -2478,16 +2478,16 @@
         <v>119.0913238525391</v>
       </c>
       <c r="F66" t="n">
-        <v>494826096.3200818</v>
+        <v>485400263.5296825</v>
       </c>
       <c r="G66" t="n">
-        <v>49.35220629730875</v>
+        <v>49.00827592529642</v>
       </c>
       <c r="H66" t="n">
-        <v>608.5433735509779</v>
+        <v>596.7649932855552</v>
       </c>
       <c r="I66" t="n">
-        <v>24.66867190488734</v>
+        <v>24.42877388011022</v>
       </c>
     </row>
     <row r="67">
@@ -2500,25 +2500,25 @@
         <v>650</v>
       </c>
       <c r="C67" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D67" t="n">
-        <v>-5.791181564331055</v>
+        <v>-9.189784049987793</v>
       </c>
       <c r="E67" t="n">
-        <v>114.8564529418945</v>
+        <v>117.3552017211914</v>
       </c>
       <c r="F67" t="n">
-        <v>476936631.3311185</v>
+        <v>467880795.5822323</v>
       </c>
       <c r="G67" t="n">
-        <v>47.56797427468587</v>
+        <v>47.23942867954186</v>
       </c>
       <c r="H67" t="n">
-        <v>750.9843119148078</v>
+        <v>732.6056884215355</v>
       </c>
       <c r="I67" t="n">
-        <v>27.40409297741503</v>
+        <v>27.06668964652928</v>
       </c>
     </row>
     <row r="68">
@@ -2531,25 +2531,25 @@
         <v>600</v>
       </c>
       <c r="C68" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D68" t="n">
-        <v>-7.655652046203613</v>
+        <v>-6.82654857635498</v>
       </c>
       <c r="E68" t="n">
-        <v>114.9189147949219</v>
+        <v>132.5256805419922</v>
       </c>
       <c r="F68" t="n">
-        <v>434971300.7473565</v>
+        <v>426225859.3938842</v>
       </c>
       <c r="G68" t="n">
-        <v>43.38250049368125</v>
+        <v>43.03375192212842</v>
       </c>
       <c r="H68" t="n">
-        <v>809.973580038239</v>
+        <v>791.3816306882889</v>
       </c>
       <c r="I68" t="n">
-        <v>28.46003478631463</v>
+        <v>28.13150601528985</v>
       </c>
     </row>
     <row r="69">
@@ -2562,25 +2562,25 @@
         <v>550</v>
       </c>
       <c r="C69" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D69" t="n">
-        <v>-4.89570140838623</v>
+        <v>-5.642542839050293</v>
       </c>
       <c r="E69" t="n">
-        <v>118.9282073974609</v>
+        <v>128.0203857421875</v>
       </c>
       <c r="F69" t="n">
-        <v>384949060.2008683</v>
+        <v>376152582.7525846</v>
       </c>
       <c r="G69" t="n">
-        <v>38.39345898341495</v>
+        <v>37.97812022494792</v>
       </c>
       <c r="H69" t="n">
-        <v>749.8189669638443</v>
+        <v>731.8469821666702</v>
       </c>
       <c r="I69" t="n">
-        <v>27.38282247986581</v>
+        <v>27.05267051820707</v>
       </c>
     </row>
     <row r="70">
@@ -2593,25 +2593,25 @@
         <v>500</v>
       </c>
       <c r="C70" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D70" t="n">
         <v>-8.479220390319824</v>
       </c>
       <c r="E70" t="n">
-        <v>131.3380889892578</v>
+        <v>133.5879058837891</v>
       </c>
       <c r="F70" t="n">
-        <v>361184774.0162191</v>
+        <v>352205976.3473574</v>
       </c>
       <c r="G70" t="n">
-        <v>36.02329305438413</v>
+        <v>35.56035908561936</v>
       </c>
       <c r="H70" t="n">
-        <v>725.6675188043481</v>
+        <v>706.7285190077654</v>
       </c>
       <c r="I70" t="n">
-        <v>26.93821669681102</v>
+        <v>26.58436606368046</v>
       </c>
     </row>
     <row r="71">
@@ -2624,25 +2624,25 @@
         <v>450</v>
       </c>
       <c r="C71" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D71" t="n">
         <v>-10.94512271881104</v>
       </c>
       <c r="E71" t="n">
-        <v>139.7909698486328</v>
+        <v>133.7244262695312</v>
       </c>
       <c r="F71" t="n">
-        <v>373099676.9571382</v>
+        <v>363179030.1803893</v>
       </c>
       <c r="G71" t="n">
-        <v>37.21164337043614</v>
+        <v>36.66824981085693</v>
       </c>
       <c r="H71" t="n">
-        <v>764.8233707592289</v>
+        <v>745.7641346622869</v>
       </c>
       <c r="I71" t="n">
-        <v>27.65544016571114</v>
+        <v>27.30868240436157</v>
       </c>
     </row>
     <row r="72">
@@ -2655,25 +2655,25 @@
         <v>400</v>
       </c>
       <c r="C72" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D72" t="n">
-        <v>-8.509300231933594</v>
+        <v>-8.745258331298828</v>
       </c>
       <c r="E72" t="n">
-        <v>139.2088928222656</v>
+        <v>133.2915802001953</v>
       </c>
       <c r="F72" t="n">
-        <v>409373090.4784034</v>
+        <v>398037181.6062763</v>
       </c>
       <c r="G72" t="n">
-        <v>40.82942545695533</v>
+        <v>40.18769145866931</v>
       </c>
       <c r="H72" t="n">
-        <v>819.3016539773708</v>
+        <v>802.7754258543857</v>
       </c>
       <c r="I72" t="n">
-        <v>28.62344587881359</v>
+        <v>28.33329182877248</v>
       </c>
     </row>
     <row r="73">
@@ -2686,25 +2686,25 @@
         <v>350</v>
       </c>
       <c r="C73" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D73" t="n">
-        <v>-5.738934516906738</v>
+        <v>-5.27549934387207</v>
       </c>
       <c r="E73" t="n">
-        <v>129.5653686523438</v>
+        <v>134.7029724121094</v>
       </c>
       <c r="F73" t="n">
-        <v>466342569.2067576</v>
+        <v>455176111.9500782</v>
       </c>
       <c r="G73" t="n">
-        <v>46.51135995426869</v>
+        <v>45.95670452842477</v>
       </c>
       <c r="H73" t="n">
-        <v>867.4816007377142</v>
+        <v>857.248276339919</v>
       </c>
       <c r="I73" t="n">
-        <v>29.45304060258829</v>
+        <v>29.27880250863958</v>
       </c>
     </row>
     <row r="74">
@@ -2717,25 +2717,25 @@
         <v>300</v>
       </c>
       <c r="C74" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D74" t="n">
-        <v>-5.420136451721191</v>
+        <v>-3.193296432495117</v>
       </c>
       <c r="E74" t="n">
-        <v>133.7701568603516</v>
+        <v>149.8188629150391</v>
       </c>
       <c r="F74" t="n">
-        <v>552663292.5238219</v>
+        <v>542160537.4497203</v>
       </c>
       <c r="G74" t="n">
-        <v>55.12068386939426</v>
+        <v>54.73905807535306</v>
       </c>
       <c r="H74" t="n">
-        <v>903.9253678769517</v>
+        <v>900.8690202394084</v>
       </c>
       <c r="I74" t="n">
-        <v>30.06535161738428</v>
+        <v>30.01448017606516</v>
       </c>
     </row>
     <row r="75">
@@ -2748,25 +2748,25 @@
         <v>250</v>
       </c>
       <c r="C75" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D75" t="n">
-        <v>-4.314042091369629</v>
+        <v>-5.87335205078125</v>
       </c>
       <c r="E75" t="n">
-        <v>168.4070892333984</v>
+        <v>154.9700012207031</v>
       </c>
       <c r="F75" t="n">
-        <v>593370526.130264</v>
+        <v>582965196.7388428</v>
       </c>
       <c r="G75" t="n">
-        <v>59.18067950357418</v>
+        <v>58.85888690885515</v>
       </c>
       <c r="H75" t="n">
-        <v>886.4656914189896</v>
+        <v>884.0042290190599</v>
       </c>
       <c r="I75" t="n">
-        <v>29.77357370923064</v>
+        <v>29.73220861320363</v>
       </c>
     </row>
     <row r="76">
@@ -2779,25 +2779,25 @@
         <v>200</v>
       </c>
       <c r="C76" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D76" t="n">
-        <v>-4.440022468566895</v>
+        <v>-2.776803016662598</v>
       </c>
       <c r="E76" t="n">
-        <v>148.8643646240234</v>
+        <v>142.6777648925781</v>
       </c>
       <c r="F76" t="n">
-        <v>618388394.1481723</v>
+        <v>607928662.6627564</v>
       </c>
       <c r="G76" t="n">
-        <v>61.67587325491589</v>
+        <v>61.37931493078182</v>
       </c>
       <c r="H76" t="n">
-        <v>831.5248213876281</v>
+        <v>828.1461726687463</v>
       </c>
       <c r="I76" t="n">
-        <v>28.83617210011808</v>
+        <v>28.77752895348637</v>
       </c>
     </row>
     <row r="77">
@@ -2810,25 +2810,25 @@
         <v>150</v>
       </c>
       <c r="C77" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D77" t="n">
-        <v>-1.075922966003418</v>
+        <v>-1.261675834655762</v>
       </c>
       <c r="E77" t="n">
-        <v>147.6380920410156</v>
+        <v>151.2321319580078</v>
       </c>
       <c r="F77" t="n">
-        <v>632354903.6394479</v>
+        <v>621660019.269586</v>
       </c>
       <c r="G77" t="n">
-        <v>63.06884355860989</v>
+        <v>62.76569677681254</v>
       </c>
       <c r="H77" t="n">
-        <v>795.9576664455182</v>
+        <v>794.2579538336554</v>
       </c>
       <c r="I77" t="n">
-        <v>28.21272171282874</v>
+        <v>28.18258245501386</v>
       </c>
     </row>
     <row r="78">
@@ -2841,25 +2841,25 @@
         <v>100</v>
       </c>
       <c r="C78" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D78" t="n">
-        <v>-19.89750671386719</v>
+        <v>-13.85577201843262</v>
       </c>
       <c r="E78" t="n">
-        <v>168.4141845703125</v>
+        <v>163.2067260742188</v>
       </c>
       <c r="F78" t="n">
-        <v>632863170.6179223</v>
+        <v>622995978.0552262</v>
       </c>
       <c r="G78" t="n">
-        <v>63.11953631099761</v>
+        <v>62.90058141061036</v>
       </c>
       <c r="H78" t="n">
-        <v>854.9545310584356</v>
+        <v>852.6120465842278</v>
       </c>
       <c r="I78" t="n">
-        <v>29.23960552159409</v>
+        <v>29.19952134169716</v>
       </c>
     </row>
     <row r="79">
@@ -2872,25 +2872,25 @@
         <v>1000</v>
       </c>
       <c r="C79" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D79" t="n">
-        <v>255.1848907470703</v>
+        <v>254.3196563720703</v>
       </c>
       <c r="E79" t="n">
-        <v>318.2398071289062</v>
+        <v>317.78955078125</v>
       </c>
       <c r="F79" t="n">
-        <v>2982892580.056778</v>
+        <v>2946632435.486938</v>
       </c>
       <c r="G79" t="n">
-        <v>297.5031653917632</v>
+        <v>297.5057623551161</v>
       </c>
       <c r="H79" t="n">
-        <v>10.29535471809472</v>
+        <v>10.47361501275375</v>
       </c>
       <c r="I79" t="n">
-        <v>3.208637517404345</v>
+        <v>3.236296496422068</v>
       </c>
     </row>
     <row r="80">
@@ -2903,25 +2903,25 @@
         <v>975</v>
       </c>
       <c r="C80" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D80" t="n">
-        <v>253.9454193115234</v>
+        <v>253.1016693115234</v>
       </c>
       <c r="E80" t="n">
-        <v>316.7802124023438</v>
+        <v>316.5765380859375</v>
       </c>
       <c r="F80" t="n">
-        <v>2964174687.582321</v>
+        <v>2928093826.634644</v>
       </c>
       <c r="G80" t="n">
-        <v>295.636308939122</v>
+        <v>295.63401788737</v>
       </c>
       <c r="H80" t="n">
-        <v>10.29164871898972</v>
+        <v>10.44498327302808</v>
       </c>
       <c r="I80" t="n">
-        <v>3.208059961875669</v>
+        <v>3.231869934423117</v>
       </c>
     </row>
     <row r="81">
@@ -2934,25 +2934,25 @@
         <v>950</v>
       </c>
       <c r="C81" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D81" t="n">
-        <v>252.6427001953125</v>
+        <v>251.9278564453125</v>
       </c>
       <c r="E81" t="n">
-        <v>315.1768798828125</v>
+        <v>314.1771240234375</v>
       </c>
       <c r="F81" t="n">
-        <v>2949466694.461182</v>
+        <v>2913503548.240021</v>
       </c>
       <c r="G81" t="n">
-        <v>294.1693856783398</v>
+        <v>294.160915289133</v>
       </c>
       <c r="H81" t="n">
-        <v>10.57754093144271</v>
+        <v>10.722842444887</v>
       </c>
       <c r="I81" t="n">
-        <v>3.252313166262239</v>
+        <v>3.274575154869255</v>
       </c>
     </row>
     <row r="82">
@@ -2965,25 +2965,25 @@
         <v>925</v>
       </c>
       <c r="C82" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D82" t="n">
-        <v>251.3966522216797</v>
+        <v>250.6466522216797</v>
       </c>
       <c r="E82" t="n">
-        <v>312.859130859375</v>
+        <v>311.7510986328125</v>
       </c>
       <c r="F82" t="n">
-        <v>2937569284.775055</v>
+        <v>2901670959.49234</v>
       </c>
       <c r="G82" t="n">
-        <v>292.982780077706</v>
+        <v>292.9662419075396</v>
       </c>
       <c r="H82" t="n">
-        <v>10.77418475424225</v>
+        <v>10.96182917689805</v>
       </c>
       <c r="I82" t="n">
-        <v>3.28240533058339</v>
+        <v>3.310865321467796</v>
       </c>
     </row>
     <row r="83">
@@ -2996,25 +2996,25 @@
         <v>900</v>
       </c>
       <c r="C83" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D83" t="n">
-        <v>250.0228271484375</v>
+        <v>249.2161865234375</v>
       </c>
       <c r="E83" t="n">
-        <v>310.3804931640625</v>
+        <v>309.3198547363281</v>
       </c>
       <c r="F83" t="n">
-        <v>2926298693.782501</v>
+        <v>2890517331.167633</v>
       </c>
       <c r="G83" t="n">
-        <v>291.8586911586017</v>
+        <v>291.8401195388983</v>
       </c>
       <c r="H83" t="n">
-        <v>10.51822467950567</v>
+        <v>10.74370414270511</v>
       </c>
       <c r="I83" t="n">
-        <v>3.243181259119766</v>
+        <v>3.277759012298664</v>
       </c>
     </row>
     <row r="84">
@@ -3027,25 +3027,25 @@
         <v>875</v>
       </c>
       <c r="C84" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D84" t="n">
-        <v>248.6092681884766</v>
+        <v>247.9276275634766</v>
       </c>
       <c r="E84" t="n">
-        <v>307.8746643066406</v>
+        <v>306.8099365234375</v>
       </c>
       <c r="F84" t="n">
-        <v>2915426337.656647</v>
+        <v>2879879374.901581</v>
       </c>
       <c r="G84" t="n">
-        <v>290.774320777872</v>
+        <v>290.7660618278929</v>
       </c>
       <c r="H84" t="n">
-        <v>10.06184956860948</v>
+        <v>10.30541099230571</v>
       </c>
       <c r="I84" t="n">
-        <v>3.172041861106104</v>
+        <v>3.210204197914162</v>
       </c>
     </row>
     <row r="85">
@@ -3058,25 +3058,25 @@
         <v>850</v>
       </c>
       <c r="C85" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D85" t="n">
         <v>247.3075866699219</v>
       </c>
       <c r="E85" t="n">
-        <v>305.3089599609375</v>
+        <v>304.2629699707031</v>
       </c>
       <c r="F85" t="n">
-        <v>2904454260.914337</v>
+        <v>2869131315.764175</v>
       </c>
       <c r="G85" t="n">
-        <v>289.6800046152406</v>
+        <v>289.6808876171564</v>
       </c>
       <c r="H85" t="n">
-        <v>9.398639052206656</v>
+        <v>9.655725942591474</v>
       </c>
       <c r="I85" t="n">
-        <v>3.065719989204275</v>
+        <v>3.107366399797661</v>
       </c>
     </row>
     <row r="86">
@@ -3089,25 +3089,25 @@
         <v>825</v>
       </c>
       <c r="C86" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D86" t="n">
         <v>247.0019073486328</v>
       </c>
       <c r="E86" t="n">
-        <v>302.8648681640625</v>
+        <v>302.1187133789062</v>
       </c>
       <c r="F86" t="n">
-        <v>2892697740.646317</v>
+        <v>2857589458.447571</v>
       </c>
       <c r="G86" t="n">
-        <v>288.5074508273095</v>
+        <v>288.5155678376628</v>
       </c>
       <c r="H86" t="n">
-        <v>8.455037033638115</v>
+        <v>8.730867258283723</v>
       </c>
       <c r="I86" t="n">
-        <v>2.907754637798402</v>
+        <v>2.954804098122873</v>
       </c>
     </row>
     <row r="87">
@@ -3120,25 +3120,25 @@
         <v>800</v>
       </c>
       <c r="C87" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D87" t="n">
         <v>246.7183990478516</v>
       </c>
       <c r="E87" t="n">
-        <v>301.2190551757812</v>
+        <v>300.1513977050781</v>
       </c>
       <c r="F87" t="n">
-        <v>2879884617.562988</v>
+        <v>2844960479.480789</v>
       </c>
       <c r="G87" t="n">
-        <v>287.2295152082643</v>
+        <v>287.2404871828671</v>
       </c>
       <c r="H87" t="n">
-        <v>7.488181342029197</v>
+        <v>7.793389339404394</v>
       </c>
       <c r="I87" t="n">
-        <v>2.736454154929184</v>
+        <v>2.791664259792784</v>
       </c>
     </row>
     <row r="88">
@@ -3151,25 +3151,25 @@
         <v>775</v>
       </c>
       <c r="C88" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D88" t="n">
-        <v>246.04736328125</v>
+        <v>245.77685546875</v>
       </c>
       <c r="E88" t="n">
-        <v>299.0550537109375</v>
+        <v>297.8041381835938</v>
       </c>
       <c r="F88" t="n">
-        <v>2866125498.536865</v>
+        <v>2831397659.48967</v>
       </c>
       <c r="G88" t="n">
-        <v>285.8572292967155</v>
+        <v>285.8711215801037</v>
       </c>
       <c r="H88" t="n">
-        <v>6.661261281562805</v>
+        <v>6.984014800767743</v>
       </c>
       <c r="I88" t="n">
-        <v>2.580941936883278</v>
+        <v>2.642728665748291</v>
       </c>
     </row>
     <row r="89">
@@ -3182,25 +3182,25 @@
         <v>750</v>
       </c>
       <c r="C89" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D89" t="n">
-        <v>246.3654022216797</v>
+        <v>244.6638641357422</v>
       </c>
       <c r="E89" t="n">
         <v>297.671630859375</v>
       </c>
       <c r="F89" t="n">
-        <v>2851552502.29895</v>
+        <v>2817037931.251205</v>
       </c>
       <c r="G89" t="n">
-        <v>284.4037701480342</v>
+        <v>284.4212964015895</v>
       </c>
       <c r="H89" t="n">
-        <v>5.974969541316645</v>
+        <v>6.28295059186824</v>
       </c>
       <c r="I89" t="n">
-        <v>2.444375081961982</v>
+        <v>2.506581455262972</v>
       </c>
     </row>
     <row r="90">
@@ -3213,25 +3213,25 @@
         <v>725</v>
       </c>
       <c r="C90" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D90" t="n">
-        <v>242.462158203125</v>
+        <v>241.5117797851562</v>
       </c>
       <c r="E90" t="n">
-        <v>294.1692504882812</v>
+        <v>294.9127807617188</v>
       </c>
       <c r="F90" t="n">
-        <v>2819645475.68222</v>
+        <v>2785567990.744934</v>
       </c>
       <c r="G90" t="n">
-        <v>281.2214760620246</v>
+        <v>281.2439443406974</v>
       </c>
       <c r="H90" t="n">
-        <v>4.945534566297511</v>
+        <v>5.183560536247198</v>
       </c>
       <c r="I90" t="n">
-        <v>2.223855788107114</v>
+        <v>2.276743405886398</v>
       </c>
     </row>
     <row r="91">
@@ -3244,25 +3244,25 @@
         <v>700</v>
       </c>
       <c r="C91" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D91" t="n">
-        <v>239.9819946289062</v>
+        <v>239.3909912109375</v>
       </c>
       <c r="E91" t="n">
-        <v>289.8150634765625</v>
+        <v>292.1351928710938</v>
       </c>
       <c r="F91" t="n">
-        <v>2783950845.061508</v>
+        <v>2750267628.544312</v>
       </c>
       <c r="G91" t="n">
-        <v>277.661419736782</v>
+        <v>277.6798550293093</v>
       </c>
       <c r="H91" t="n">
-        <v>4.40748699557196</v>
+        <v>4.577352300679132</v>
       </c>
       <c r="I91" t="n">
-        <v>2.099401580349019</v>
+        <v>2.139474772153</v>
       </c>
     </row>
     <row r="92">
@@ -3275,25 +3275,25 @@
         <v>650</v>
       </c>
       <c r="C92" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D92" t="n">
-        <v>238.6626434326172</v>
+        <v>238.0354156494141</v>
       </c>
       <c r="E92" t="n">
-        <v>286.2237548828125</v>
+        <v>288.7566223144531</v>
       </c>
       <c r="F92" t="n">
-        <v>2747194936.990646</v>
+        <v>2713834135.602066</v>
       </c>
       <c r="G92" t="n">
-        <v>273.9955153488576</v>
+        <v>274.0013595500276</v>
       </c>
       <c r="H92" t="n">
-        <v>4.273986207056101</v>
+        <v>4.409659398916618</v>
       </c>
       <c r="I92" t="n">
-        <v>2.067362137376057</v>
+        <v>2.099918902938068</v>
       </c>
     </row>
     <row r="93">
@@ -3306,25 +3306,25 @@
         <v>600</v>
       </c>
       <c r="C93" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D93" t="n">
-        <v>236.7375946044922</v>
+        <v>234.7569122314453</v>
       </c>
       <c r="E93" t="n">
-        <v>281.2777099609375</v>
+        <v>283.3309326171875</v>
       </c>
       <c r="F93" t="n">
-        <v>2709923650.035248</v>
+        <v>2676915473.054916</v>
       </c>
       <c r="G93" t="n">
-        <v>270.2782088921709</v>
+        <v>270.2738790831924</v>
       </c>
       <c r="H93" t="n">
-        <v>4.871282870012011</v>
+        <v>5.008298228264893</v>
       </c>
       <c r="I93" t="n">
-        <v>2.207098291878278</v>
+        <v>2.23792274850248</v>
       </c>
     </row>
     <row r="94">
@@ -3337,25 +3337,25 @@
         <v>550</v>
       </c>
       <c r="C94" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D94" t="n">
-        <v>233.0751647949219</v>
+        <v>231.8300323486328</v>
       </c>
       <c r="E94" t="n">
-        <v>278.5971069335938</v>
+        <v>279.7101440429688</v>
       </c>
       <c r="F94" t="n">
-        <v>2667786780.278778</v>
+        <v>2635290789.360687</v>
       </c>
       <c r="G94" t="n">
-        <v>266.0756264002401</v>
+        <v>266.0712567587726</v>
       </c>
       <c r="H94" t="n">
-        <v>5.68423344348288</v>
+        <v>5.856825407494704</v>
       </c>
       <c r="I94" t="n">
-        <v>2.384163048846047</v>
+        <v>2.420087892514382</v>
       </c>
     </row>
     <row r="95">
@@ -3368,25 +3368,25 @@
         <v>500</v>
       </c>
       <c r="C95" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D95" t="n">
-        <v>229.6830139160156</v>
+        <v>228.6268768310547</v>
       </c>
       <c r="E95" t="n">
-        <v>274.2037963867188</v>
+        <v>276.3261108398438</v>
       </c>
       <c r="F95" t="n">
-        <v>2618367403.070099</v>
+        <v>2586434360.782028</v>
       </c>
       <c r="G95" t="n">
-        <v>261.1467123489696</v>
+        <v>261.1384837209135</v>
       </c>
       <c r="H95" t="n">
-        <v>6.68986304673547</v>
+        <v>6.899376076590056</v>
       </c>
       <c r="I95" t="n">
-        <v>2.586476956544455</v>
+        <v>2.626666342836497</v>
       </c>
     </row>
     <row r="96">
@@ -3399,25 +3399,25 @@
         <v>450</v>
       </c>
       <c r="C96" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D96" t="n">
-        <v>225.9030609130859</v>
+        <v>225.0690765380859</v>
       </c>
       <c r="E96" t="n">
-        <v>267.074951171875</v>
+        <v>270.71875</v>
       </c>
       <c r="F96" t="n">
-        <v>2559050547.163849</v>
+        <v>2527744478.127563</v>
       </c>
       <c r="G96" t="n">
-        <v>255.2306587467777</v>
+        <v>255.2128792677195</v>
       </c>
       <c r="H96" t="n">
-        <v>7.493912165690227</v>
+        <v>7.705515311810009</v>
       </c>
       <c r="I96" t="n">
-        <v>2.737501080491152</v>
+        <v>2.775880997415057</v>
       </c>
     </row>
     <row r="97">
@@ -3430,25 +3430,25 @@
         <v>400</v>
       </c>
       <c r="C97" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D97" t="n">
         <v>221.6041412353516</v>
       </c>
       <c r="E97" t="n">
-        <v>261.0946044921875</v>
+        <v>263.681640625</v>
       </c>
       <c r="F97" t="n">
-        <v>2488197158.048065</v>
+        <v>2457732863.997284</v>
       </c>
       <c r="G97" t="n">
-        <v>248.1639920885112</v>
+        <v>248.1441799672258</v>
       </c>
       <c r="H97" t="n">
-        <v>7.876223627061692</v>
+        <v>8.092607266499595</v>
       </c>
       <c r="I97" t="n">
-        <v>2.80646105033754</v>
+        <v>2.844750826785994</v>
       </c>
     </row>
     <row r="98">
@@ -3461,25 +3461,25 @@
         <v>350</v>
       </c>
       <c r="C98" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D98" t="n">
-        <v>216.825927734375</v>
+        <v>216.7074432373047</v>
       </c>
       <c r="E98" t="n">
-        <v>253.9608917236328</v>
+        <v>255.7990875244141</v>
       </c>
       <c r="F98" t="n">
-        <v>2403975695.42659</v>
+        <v>2374541560.531219</v>
       </c>
       <c r="G98" t="n">
-        <v>239.764041017079</v>
+        <v>239.7447977229657</v>
       </c>
       <c r="H98" t="n">
-        <v>7.575955226003828</v>
+        <v>7.722623300677319</v>
       </c>
       <c r="I98" t="n">
-        <v>2.752445317531999</v>
+        <v>2.778960831080085</v>
       </c>
     </row>
     <row r="99">
@@ -3492,25 +3492,25 @@
         <v>300</v>
       </c>
       <c r="C99" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D99" t="n">
-        <v>210.1175231933594</v>
+        <v>209.8344573974609</v>
       </c>
       <c r="E99" t="n">
-        <v>243.81591796875</v>
+        <v>245.8572235107422</v>
       </c>
       <c r="F99" t="n">
-        <v>2304446570.033173</v>
+        <v>2276344154.098923</v>
       </c>
       <c r="G99" t="n">
-        <v>229.8373577529269</v>
+        <v>229.8303292911035</v>
       </c>
       <c r="H99" t="n">
-        <v>6.10071474178661</v>
+        <v>6.110700129219928</v>
       </c>
       <c r="I99" t="n">
-        <v>2.469962498052675</v>
+        <v>2.471983035787246</v>
       </c>
     </row>
     <row r="100">
@@ -3523,25 +3523,25 @@
         <v>250</v>
       </c>
       <c r="C100" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D100" t="n">
-        <v>205.1709289550781</v>
+        <v>206.8453216552734</v>
       </c>
       <c r="E100" t="n">
-        <v>238.6356811523438</v>
+        <v>239.6231536865234</v>
       </c>
       <c r="F100" t="n">
-        <v>2248466244.028961</v>
+        <v>2221121307.007431</v>
       </c>
       <c r="G100" t="n">
-        <v>224.2540778529853</v>
+        <v>224.25477292869</v>
       </c>
       <c r="H100" t="n">
-        <v>4.79171467876384</v>
+        <v>4.74228599998435</v>
       </c>
       <c r="I100" t="n">
-        <v>2.188998556135622</v>
+        <v>2.177679039708182</v>
       </c>
     </row>
     <row r="101">
@@ -3554,25 +3554,25 @@
         <v>200</v>
       </c>
       <c r="C101" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D101" t="n">
-        <v>202.6686401367188</v>
+        <v>203.9869079589844</v>
       </c>
       <c r="E101" t="n">
-        <v>235.3539276123047</v>
+        <v>235.3334808349609</v>
       </c>
       <c r="F101" t="n">
-        <v>2188973182.29628</v>
+        <v>2162443892.994141</v>
       </c>
       <c r="G101" t="n">
-        <v>218.3204501043177</v>
+        <v>218.3304273676994</v>
       </c>
       <c r="H101" t="n">
-        <v>3.513912503862053</v>
+        <v>3.456563859657978</v>
       </c>
       <c r="I101" t="n">
-        <v>1.874543278738065</v>
+        <v>1.85918365409606</v>
       </c>
     </row>
     <row r="102">
@@ -3585,25 +3585,25 @@
         <v>150</v>
       </c>
       <c r="C102" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D102" t="n">
         <v>199.7282409667969</v>
       </c>
       <c r="E102" t="n">
-        <v>231.593505859375</v>
+        <v>231.5911560058594</v>
       </c>
       <c r="F102" t="n">
-        <v>2127541516.277298</v>
+        <v>2101854445.244751</v>
       </c>
       <c r="G102" t="n">
-        <v>212.1934728145124</v>
+        <v>212.2130339574209</v>
       </c>
       <c r="H102" t="n">
-        <v>3.717591481198834</v>
+        <v>3.727950877535779</v>
       </c>
       <c r="I102" t="n">
-        <v>1.928105671688882</v>
+        <v>1.930790221006875</v>
       </c>
     </row>
     <row r="103">
@@ -3616,25 +3616,25 @@
         <v>100</v>
       </c>
       <c r="C103" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D103" t="n">
-        <v>197.075439453125</v>
+        <v>197.5082550048828</v>
       </c>
       <c r="E103" t="n">
-        <v>229.3795166015625</v>
+        <v>228.7249298095703</v>
       </c>
       <c r="F103" t="n">
-        <v>2067850418.73085</v>
+        <v>2042909904.433975</v>
       </c>
       <c r="G103" t="n">
-        <v>206.2400936735711</v>
+        <v>206.2617180282992</v>
       </c>
       <c r="H103" t="n">
-        <v>7.949036296630696</v>
+        <v>7.957001502644427</v>
       </c>
       <c r="I103" t="n">
-        <v>2.81940353561364</v>
+        <v>2.820815751275582</v>
       </c>
     </row>
     <row r="104">
@@ -3647,25 +3647,25 @@
         <v>1000</v>
       </c>
       <c r="C104" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D104" t="n">
-        <v>-35.444091796875</v>
+        <v>-38.69720458984375</v>
       </c>
       <c r="E104" t="n">
-        <v>31.78263854980469</v>
+        <v>30.55911254882812</v>
       </c>
       <c r="F104" t="n">
-        <v>-28661084.70574951</v>
+        <v>-28485397.36917114</v>
       </c>
       <c r="G104" t="n">
-        <v>-2.85855530987966</v>
+        <v>-2.876018657177108</v>
       </c>
       <c r="H104" t="n">
-        <v>21.09356699685789</v>
+        <v>20.81096202419509</v>
       </c>
       <c r="I104" t="n">
-        <v>4.592773344816603</v>
+        <v>4.561903333499636</v>
       </c>
     </row>
     <row r="105">
@@ -3678,25 +3678,25 @@
         <v>975</v>
       </c>
       <c r="C105" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D105" t="n">
         <v>-44.34205627441406</v>
       </c>
       <c r="E105" t="n">
-        <v>35.90019226074219</v>
+        <v>36.06578063964844</v>
       </c>
       <c r="F105" t="n">
-        <v>-31036257.70367432</v>
+        <v>-30828405.46591187</v>
       </c>
       <c r="G105" t="n">
-        <v>-3.095446671626996</v>
+        <v>-3.112579689231937</v>
       </c>
       <c r="H105" t="n">
-        <v>25.17002160117967</v>
+        <v>24.87714970616775</v>
       </c>
       <c r="I105" t="n">
-        <v>5.016973350654721</v>
+        <v>4.987699841226188</v>
       </c>
     </row>
     <row r="106">
@@ -3709,25 +3709,25 @@
         <v>950</v>
       </c>
       <c r="C106" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D106" t="n">
-        <v>-55.71876525878906</v>
+        <v>-55.7569580078125</v>
       </c>
       <c r="E106" t="n">
-        <v>44.95748901367188</v>
+        <v>46.89558410644531</v>
       </c>
       <c r="F106" t="n">
-        <v>-32511455.06626892</v>
+        <v>-32300441.23620605</v>
       </c>
       <c r="G106" t="n">
-        <v>-3.242577643718893</v>
+        <v>-3.26120329045931</v>
       </c>
       <c r="H106" t="n">
-        <v>28.19293071790275</v>
+        <v>27.89172639003009</v>
       </c>
       <c r="I106" t="n">
-        <v>5.309701565804122</v>
+        <v>5.281261817977791</v>
       </c>
     </row>
     <row r="107">
@@ -3740,25 +3740,25 @@
         <v>925</v>
       </c>
       <c r="C107" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D107" t="n">
-        <v>-58.72221374511719</v>
+        <v>-61.9556884765625</v>
       </c>
       <c r="E107" t="n">
-        <v>49.02644348144531</v>
+        <v>51.88597106933594</v>
       </c>
       <c r="F107" t="n">
-        <v>-32494862.96014404</v>
+        <v>-32347670.70326233</v>
       </c>
       <c r="G107" t="n">
-        <v>-3.240922805684942</v>
+        <v>-3.265971797868959</v>
       </c>
       <c r="H107" t="n">
-        <v>29.73806395968585</v>
+        <v>29.44244765134103</v>
       </c>
       <c r="I107" t="n">
-        <v>5.453261772525307</v>
+        <v>5.426089535875817</v>
       </c>
     </row>
     <row r="108">
@@ -3771,25 +3771,25 @@
         <v>900</v>
       </c>
       <c r="C108" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D108" t="n">
-        <v>-57.55891418457031</v>
+        <v>-62.35000610351562</v>
       </c>
       <c r="E108" t="n">
-        <v>50.91188049316406</v>
+        <v>51.50082397460938</v>
       </c>
       <c r="F108" t="n">
-        <v>-31972289.9831543</v>
+        <v>-31893965.07331848</v>
       </c>
       <c r="G108" t="n">
-        <v>-3.188803223557825</v>
+        <v>-3.220163560066508</v>
       </c>
       <c r="H108" t="n">
-        <v>30.37371641299665</v>
+        <v>30.12949181280628</v>
       </c>
       <c r="I108" t="n">
-        <v>5.511235470654166</v>
+        <v>5.489033777706809</v>
       </c>
     </row>
     <row r="109">
@@ -3802,25 +3802,25 @@
         <v>875</v>
       </c>
       <c r="C109" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D109" t="n">
-        <v>-55.08590698242188</v>
+        <v>-63.30732727050781</v>
       </c>
       <c r="E109" t="n">
-        <v>52.4219970703125</v>
+        <v>51.68013000488281</v>
       </c>
       <c r="F109" t="n">
-        <v>-31157462.40396118</v>
+        <v>-31132721.64068604</v>
       </c>
       <c r="G109" t="n">
-        <v>-3.107535200136789</v>
+        <v>-3.143304870453351</v>
       </c>
       <c r="H109" t="n">
-        <v>30.78586801517007</v>
+        <v>30.61963203249524</v>
       </c>
       <c r="I109" t="n">
-        <v>5.548501420669375</v>
+        <v>5.533500883933717</v>
       </c>
     </row>
     <row r="110">
@@ -3833,25 +3833,25 @@
         <v>850</v>
       </c>
       <c r="C110" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D110" t="n">
-        <v>-54.52687072753906</v>
+        <v>-63.0902099609375</v>
       </c>
       <c r="E110" t="n">
-        <v>52.21392822265625</v>
+        <v>50.84359741210938</v>
       </c>
       <c r="F110" t="n">
-        <v>-30273145.1541748</v>
+        <v>-30294053.06414795</v>
       </c>
       <c r="G110" t="n">
-        <v>-3.019336522524002</v>
+        <v>-3.058628976975302</v>
       </c>
       <c r="H110" t="n">
-        <v>31.45466007862744</v>
+        <v>31.36525652958391</v>
       </c>
       <c r="I110" t="n">
-        <v>5.608445424413743</v>
+        <v>5.600469313332939</v>
       </c>
     </row>
     <row r="111">
@@ -3864,25 +3864,25 @@
         <v>825</v>
       </c>
       <c r="C111" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D111" t="n">
-        <v>-53.82025146484375</v>
+        <v>-62.351318359375</v>
       </c>
       <c r="E111" t="n">
-        <v>53.10092163085938</v>
+        <v>50.95205688476562</v>
       </c>
       <c r="F111" t="n">
-        <v>-29413944.10871887</v>
+        <v>-29476024.06838989</v>
       </c>
       <c r="G111" t="n">
-        <v>-2.933642846378917</v>
+        <v>-2.976036951895874</v>
       </c>
       <c r="H111" t="n">
-        <v>32.57910105197477</v>
+        <v>32.54356938871108</v>
       </c>
       <c r="I111" t="n">
-        <v>5.707810530490195</v>
+        <v>5.704697133828498</v>
       </c>
     </row>
     <row r="112">
@@ -3895,25 +3895,25 @@
         <v>800</v>
       </c>
       <c r="C112" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D112" t="n">
-        <v>-53.17196655273438</v>
+        <v>-61.39985656738281</v>
       </c>
       <c r="E112" t="n">
-        <v>55.35334777832031</v>
+        <v>50.50736999511719</v>
       </c>
       <c r="F112" t="n">
-        <v>-28605625.79428101</v>
+        <v>-28722261.02346802</v>
       </c>
       <c r="G112" t="n">
-        <v>-2.853024034023006</v>
+        <v>-2.899933517136269</v>
       </c>
       <c r="H112" t="n">
-        <v>34.16042425945646</v>
+        <v>34.17599223637693</v>
       </c>
       <c r="I112" t="n">
-        <v>5.844691973017608</v>
+        <v>5.846023626053604</v>
       </c>
     </row>
     <row r="113">
@@ -3926,25 +3926,25 @@
         <v>775</v>
       </c>
       <c r="C113" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D113" t="n">
-        <v>-51.88919067382812</v>
+        <v>-60.44361877441406</v>
       </c>
       <c r="E113" t="n">
-        <v>57.48287963867188</v>
+        <v>49.86827087402344</v>
       </c>
       <c r="F113" t="n">
-        <v>-27833527.2855072</v>
+        <v>-28023921.97550964</v>
       </c>
       <c r="G113" t="n">
-        <v>-2.776017657095372</v>
+        <v>-2.829425947768919</v>
       </c>
       <c r="H113" t="n">
-        <v>36.08159037987387</v>
+        <v>36.17797611460743</v>
       </c>
       <c r="I113" t="n">
-        <v>6.006795350257396</v>
+        <v>6.014813057328335</v>
       </c>
     </row>
     <row r="114">
@@ -3957,25 +3957,25 @@
         <v>750</v>
       </c>
       <c r="C114" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D114" t="n">
-        <v>-50.31416320800781</v>
+        <v>-59.44984436035156</v>
       </c>
       <c r="E114" t="n">
-        <v>58.69093322753906</v>
+        <v>50.59733581542969</v>
       </c>
       <c r="F114" t="n">
-        <v>-26999438.57720947</v>
+        <v>-27282928.5418396</v>
       </c>
       <c r="G114" t="n">
-        <v>-2.692828596719821</v>
+        <v>-2.754611792555941</v>
       </c>
       <c r="H114" t="n">
-        <v>38.14796134749733</v>
+        <v>38.35974345009902</v>
       </c>
       <c r="I114" t="n">
-        <v>6.176403593313615</v>
+        <v>6.193524315775229</v>
       </c>
     </row>
     <row r="115">
@@ -3988,25 +3988,25 @@
         <v>725</v>
       </c>
       <c r="C115" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D115" t="n">
-        <v>-48.82179260253906</v>
+        <v>-57.47085571289062</v>
       </c>
       <c r="E115" t="n">
-        <v>56.70549011230469</v>
+        <v>53.33103942871094</v>
       </c>
       <c r="F115" t="n">
-        <v>-24917005.25315857</v>
+        <v>-25333419.78370667</v>
       </c>
       <c r="G115" t="n">
-        <v>-2.485134055600745</v>
+        <v>-2.557780290152926</v>
       </c>
       <c r="H115" t="n">
-        <v>42.25084711657594</v>
+        <v>42.79226711108313</v>
       </c>
       <c r="I115" t="n">
-        <v>6.500065162486907</v>
+        <v>6.541579863540851</v>
       </c>
     </row>
     <row r="116">
@@ -4019,25 +4019,25 @@
         <v>700</v>
       </c>
       <c r="C116" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D116" t="n">
-        <v>-48.69514465332031</v>
+        <v>-55.18896484375</v>
       </c>
       <c r="E116" t="n">
-        <v>54.64736938476562</v>
+        <v>53.3035888671875</v>
       </c>
       <c r="F116" t="n">
-        <v>-22558606.70152283</v>
+        <v>-23018280.27198792</v>
       </c>
       <c r="G116" t="n">
-        <v>-2.24991571785099</v>
+        <v>-2.324033000502087</v>
       </c>
       <c r="H116" t="n">
-        <v>45.94430222578744</v>
+        <v>46.95038988771768</v>
       </c>
       <c r="I116" t="n">
-        <v>6.778222645044012</v>
+        <v>6.852035455812942</v>
       </c>
     </row>
     <row r="117">
@@ -4050,25 +4050,25 @@
         <v>650</v>
       </c>
       <c r="C117" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D117" t="n">
-        <v>-46.45986938476562</v>
+        <v>-52.69477844238281</v>
       </c>
       <c r="E117" t="n">
-        <v>55.64677429199219</v>
+        <v>56.28604125976562</v>
       </c>
       <c r="F117" t="n">
-        <v>-19913107.31484985</v>
+        <v>-20272360.38645935</v>
       </c>
       <c r="G117" t="n">
-        <v>-1.986062957332828</v>
+        <v>-2.046792113898176</v>
       </c>
       <c r="H117" t="n">
-        <v>48.61532829265593</v>
+        <v>49.88764361165846</v>
       </c>
       <c r="I117" t="n">
-        <v>6.972469310987028</v>
+        <v>7.063118547189935</v>
       </c>
     </row>
     <row r="118">
@@ -4081,25 +4081,25 @@
         <v>600</v>
       </c>
       <c r="C118" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D118" t="n">
-        <v>-42.60932922363281</v>
+        <v>-49.88926696777344</v>
       </c>
       <c r="E118" t="n">
-        <v>56.51473999023438</v>
+        <v>59.70863342285156</v>
       </c>
       <c r="F118" t="n">
-        <v>-16863510.49951172</v>
+        <v>-17092248.7870636</v>
       </c>
       <c r="G118" t="n">
-        <v>-1.681906947224517</v>
+        <v>-1.725713205528586</v>
       </c>
       <c r="H118" t="n">
-        <v>51.42436839154606</v>
+        <v>52.7351273484099</v>
       </c>
       <c r="I118" t="n">
-        <v>7.171078607263071</v>
+        <v>7.261895575427252</v>
       </c>
     </row>
     <row r="119">
@@ -4112,25 +4112,25 @@
         <v>550</v>
       </c>
       <c r="C119" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D119" t="n">
-        <v>-44.61569213867188</v>
+        <v>-47.72129821777344</v>
       </c>
       <c r="E119" t="n">
-        <v>63.27864074707031</v>
+        <v>63.10870361328125</v>
       </c>
       <c r="F119" t="n">
-        <v>-13154174.16743469</v>
+        <v>-13342884.38479614</v>
       </c>
       <c r="G119" t="n">
-        <v>-1.311950849015109</v>
+        <v>-1.347159877529471</v>
       </c>
       <c r="H119" t="n">
-        <v>56.20833926221006</v>
+        <v>57.59203663136957</v>
       </c>
       <c r="I119" t="n">
-        <v>7.497222103033233</v>
+        <v>7.588941733296519</v>
       </c>
     </row>
     <row r="120">
@@ -4143,25 +4143,25 @@
         <v>500</v>
       </c>
       <c r="C120" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D120" t="n">
-        <v>-44.61308288574219</v>
+        <v>-45.96467590332031</v>
       </c>
       <c r="E120" t="n">
-        <v>70.44790649414062</v>
+        <v>68.8433837890625</v>
       </c>
       <c r="F120" t="n">
-        <v>-8158247.426391602</v>
+        <v>-8081665.683181763</v>
       </c>
       <c r="G120" t="n">
-        <v>-0.8136747697949304</v>
+        <v>-0.8159626837803535</v>
       </c>
       <c r="H120" t="n">
-        <v>63.64295968479935</v>
+        <v>64.79807183038747</v>
       </c>
       <c r="I120" t="n">
-        <v>7.97765377067715</v>
+        <v>8.049724953710374</v>
       </c>
     </row>
     <row r="121">
@@ -4174,25 +4174,25 @@
         <v>450</v>
       </c>
       <c r="C121" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D121" t="n">
-        <v>-48.41604614257812</v>
+        <v>-44.16006469726562</v>
       </c>
       <c r="E121" t="n">
-        <v>77.19099426269531</v>
+        <v>75.38790893554688</v>
       </c>
       <c r="F121" t="n">
-        <v>-1540757.556732178</v>
+        <v>-1392350.452362061</v>
       </c>
       <c r="G121" t="n">
-        <v>-0.15366971418742</v>
+        <v>-0.1405781996447121</v>
       </c>
       <c r="H121" t="n">
-        <v>73.77414047976907</v>
+        <v>75.03823965913674</v>
       </c>
       <c r="I121" t="n">
-        <v>8.589187416733266</v>
+        <v>8.66246152425145</v>
       </c>
     </row>
     <row r="122">
@@ -4205,25 +4205,25 @@
         <v>400</v>
       </c>
       <c r="C122" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D122" t="n">
-        <v>-51.37127685546875</v>
+        <v>-42.07801818847656</v>
       </c>
       <c r="E122" t="n">
-        <v>81.51275634765625</v>
+        <v>77.19903564453125</v>
       </c>
       <c r="F122" t="n">
-        <v>6650853.389419556</v>
+        <v>6677834.168365479</v>
       </c>
       <c r="G122" t="n">
-        <v>0.6633326151728853</v>
+        <v>0.6742253024891826</v>
       </c>
       <c r="H122" t="n">
-        <v>88.24840345671007</v>
+        <v>89.72428834889688</v>
       </c>
       <c r="I122" t="n">
-        <v>9.394062138218485</v>
+        <v>9.472290554501424</v>
       </c>
     </row>
     <row r="123">
@@ -4236,25 +4236,25 @@
         <v>350</v>
       </c>
       <c r="C123" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D123" t="n">
-        <v>-52.45257568359375</v>
+        <v>-43.08665466308594</v>
       </c>
       <c r="E123" t="n">
-        <v>84.01470947265625</v>
+        <v>84.96342468261719</v>
       </c>
       <c r="F123" t="n">
-        <v>17100744.74638367</v>
+        <v>17055716.34919739</v>
       </c>
       <c r="G123" t="n">
-        <v>1.705567852701174</v>
+        <v>1.72202472010801</v>
       </c>
       <c r="H123" t="n">
-        <v>109.7875129566108</v>
+        <v>110.8579537774895</v>
       </c>
       <c r="I123" t="n">
-        <v>10.47795366264858</v>
+        <v>10.52891037940249</v>
       </c>
     </row>
     <row r="124">
@@ -4267,25 +4267,25 @@
         <v>300</v>
       </c>
       <c r="C124" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D124" t="n">
-        <v>-48.10688781738281</v>
+        <v>-48.26020812988281</v>
       </c>
       <c r="E124" t="n">
-        <v>84.57643127441406</v>
+        <v>87.12361145019531</v>
       </c>
       <c r="F124" t="n">
-        <v>30142345.76089478</v>
+        <v>30137028.19355774</v>
       </c>
       <c r="G124" t="n">
-        <v>3.006291053239497</v>
+        <v>3.042775013219585</v>
       </c>
       <c r="H124" t="n">
-        <v>138.7934274237285</v>
+        <v>139.3159406519879</v>
       </c>
       <c r="I124" t="n">
-        <v>11.78106223664609</v>
+        <v>11.80321738561092</v>
       </c>
     </row>
     <row r="125">
@@ -4298,25 +4298,25 @@
         <v>250</v>
       </c>
       <c r="C125" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D125" t="n">
-        <v>-46.27247619628906</v>
+        <v>-47.76541137695312</v>
       </c>
       <c r="E125" t="n">
         <v>82.59519958496094</v>
       </c>
       <c r="F125" t="n">
-        <v>37796574.24908447</v>
+        <v>37787374.69078064</v>
       </c>
       <c r="G125" t="n">
-        <v>3.769696755172261</v>
+        <v>3.815189699057711</v>
       </c>
       <c r="H125" t="n">
-        <v>153.5021143108031</v>
+        <v>154.0149336731059</v>
       </c>
       <c r="I125" t="n">
-        <v>12.38959701970985</v>
+        <v>12.41027532624099</v>
       </c>
     </row>
     <row r="126">
@@ -4329,25 +4329,25 @@
         <v>200</v>
       </c>
       <c r="C126" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D126" t="n">
-        <v>-44.70292663574219</v>
+        <v>-42.19203186035156</v>
       </c>
       <c r="E126" t="n">
-        <v>83.59883117675781</v>
+        <v>84.77070617675781</v>
       </c>
       <c r="F126" t="n">
-        <v>46234103.39624023</v>
+        <v>46038909.79142761</v>
       </c>
       <c r="G126" t="n">
-        <v>4.611226096908199</v>
+        <v>4.648303191990639</v>
       </c>
       <c r="H126" t="n">
-        <v>161.9187947343962</v>
+        <v>162.6779853278291</v>
       </c>
       <c r="I126" t="n">
-        <v>12.7247316173818</v>
+        <v>12.75452803234322</v>
       </c>
     </row>
     <row r="127">
@@ -4360,25 +4360,25 @@
         <v>150</v>
       </c>
       <c r="C127" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D127" t="n">
-        <v>-42.92500305175781</v>
+        <v>-41.26174926757812</v>
       </c>
       <c r="E127" t="n">
-        <v>79.32940673828125</v>
+        <v>79.56495666503906</v>
       </c>
       <c r="F127" t="n">
-        <v>52524229.86404419</v>
+        <v>51891153.00796509</v>
       </c>
       <c r="G127" t="n">
-        <v>5.238581083607199</v>
+        <v>5.239172979024613</v>
       </c>
       <c r="H127" t="n">
-        <v>155.1328340536776</v>
+        <v>155.8666527236148</v>
       </c>
       <c r="I127" t="n">
-        <v>12.45523319948999</v>
+        <v>12.4846566922609</v>
       </c>
     </row>
     <row r="128">
@@ -4391,25 +4391,25 @@
         <v>100</v>
       </c>
       <c r="C128" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D128" t="n">
-        <v>-38.6629638671875</v>
+        <v>-41.47625732421875</v>
       </c>
       <c r="E128" t="n">
         <v>72.023681640625</v>
       </c>
       <c r="F128" t="n">
-        <v>52531240.88981628</v>
+        <v>51835718.18338013</v>
       </c>
       <c r="G128" t="n">
-        <v>5.239280338543074</v>
+        <v>5.233576020425165</v>
       </c>
       <c r="H128" t="n">
-        <v>128.9300631317917</v>
+        <v>130.229618442277</v>
       </c>
       <c r="I128" t="n">
-        <v>11.35473747524758</v>
+        <v>11.411819243323</v>
       </c>
     </row>
     <row r="129">
@@ -4422,25 +4422,25 @@
         <v>1000</v>
       </c>
       <c r="C129" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D129" t="n">
-        <v>-32.6859130859375</v>
+        <v>-37.298583984375</v>
       </c>
       <c r="E129" t="n">
         <v>34.28530883789062</v>
       </c>
       <c r="F129" t="n">
-        <v>3020644.900299072</v>
+        <v>2722053.059677124</v>
       </c>
       <c r="G129" t="n">
-        <v>0.3012684484086758</v>
+        <v>0.2748311804816246</v>
       </c>
       <c r="H129" t="n">
-        <v>14.44922339250339</v>
+        <v>14.30414320368521</v>
       </c>
       <c r="I129" t="n">
-        <v>3.801213410544506</v>
+        <v>3.782081861050235</v>
       </c>
     </row>
     <row r="130">
@@ -4453,25 +4453,25 @@
         <v>975</v>
       </c>
       <c r="C130" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D130" t="n">
-        <v>-38.95536804199219</v>
+        <v>-39.46832275390625</v>
       </c>
       <c r="E130" t="n">
-        <v>40.86978149414062</v>
+        <v>41.77491760253906</v>
       </c>
       <c r="F130" t="n">
-        <v>3610669.231277466</v>
+        <v>3317250.00680542</v>
       </c>
       <c r="G130" t="n">
-        <v>0.3601153902321367</v>
+        <v>0.334925041994276</v>
       </c>
       <c r="H130" t="n">
-        <v>17.07739181541644</v>
+        <v>16.9563766958445</v>
       </c>
       <c r="I130" t="n">
-        <v>4.132480104660691</v>
+        <v>4.117812124884343</v>
       </c>
     </row>
     <row r="131">
@@ -4484,25 +4484,25 @@
         <v>950</v>
       </c>
       <c r="C131" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D131" t="n">
-        <v>-48.9976806640625</v>
+        <v>-54.18948364257812</v>
       </c>
       <c r="E131" t="n">
-        <v>53.12228393554688</v>
+        <v>59.4952392578125</v>
       </c>
       <c r="F131" t="n">
-        <v>4672600.524200439</v>
+        <v>4336245.421279907</v>
       </c>
       <c r="G131" t="n">
-        <v>0.4660286648788342</v>
+        <v>0.4378075745995006</v>
       </c>
       <c r="H131" t="n">
-        <v>17.84978739926698</v>
+        <v>17.72748990822002</v>
       </c>
       <c r="I131" t="n">
-        <v>4.224900874490072</v>
+        <v>4.210402582677816</v>
       </c>
     </row>
     <row r="132">
@@ -4515,25 +4515,25 @@
         <v>925</v>
       </c>
       <c r="C132" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D132" t="n">
-        <v>-54.05300903320312</v>
+        <v>-61.78614807128906</v>
       </c>
       <c r="E132" t="n">
-        <v>59.66902160644531</v>
+        <v>64.50277709960938</v>
       </c>
       <c r="F132" t="n">
-        <v>5516435.754348755</v>
+        <v>5148640.639938354</v>
       </c>
       <c r="G132" t="n">
-        <v>0.5501898089028102</v>
+        <v>0.5198307872506207</v>
       </c>
       <c r="H132" t="n">
-        <v>17.27271407468447</v>
+        <v>17.07536442418462</v>
       </c>
       <c r="I132" t="n">
-        <v>4.156045485155867</v>
+        <v>4.132234797804285</v>
       </c>
     </row>
     <row r="133">
@@ -4546,25 +4546,25 @@
         <v>900</v>
       </c>
       <c r="C133" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D133" t="n">
-        <v>-56.42100524902344</v>
+        <v>-62.3619384765625</v>
       </c>
       <c r="E133" t="n">
-        <v>59.36355590820312</v>
+        <v>65.13273620605469</v>
       </c>
       <c r="F133" t="n">
-        <v>5868094.359527588</v>
+        <v>5514459.938323975</v>
       </c>
       <c r="G133" t="n">
-        <v>0.5852629955396456</v>
+        <v>0.5567656108613738</v>
       </c>
       <c r="H133" t="n">
-        <v>16.41085197056272</v>
+        <v>16.14136307614882</v>
       </c>
       <c r="I133" t="n">
-        <v>4.051030976253172</v>
+        <v>4.01763152568137</v>
       </c>
     </row>
     <row r="134">
@@ -4577,25 +4577,25 @@
         <v>875</v>
       </c>
       <c r="C134" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D134" t="n">
-        <v>-56.56988525390625</v>
+        <v>-60.04344177246094</v>
       </c>
       <c r="E134" t="n">
-        <v>60.85801696777344</v>
+        <v>66.50411987304688</v>
       </c>
       <c r="F134" t="n">
-        <v>5915523.936264038</v>
+        <v>5589507.06791687</v>
       </c>
       <c r="G134" t="n">
-        <v>0.589993453923103</v>
+        <v>0.564342719303268</v>
       </c>
       <c r="H134" t="n">
-        <v>15.74153775086646</v>
+        <v>15.45974643937352</v>
       </c>
       <c r="I134" t="n">
-        <v>3.967560680174465</v>
+        <v>3.931888406271663</v>
       </c>
     </row>
     <row r="135">
@@ -4608,25 +4608,25 @@
         <v>850</v>
       </c>
       <c r="C135" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D135" t="n">
-        <v>-54.69912719726562</v>
+        <v>-58.49705505371094</v>
       </c>
       <c r="E135" t="n">
-        <v>60.85945129394531</v>
+        <v>66.01028442382812</v>
       </c>
       <c r="F135" t="n">
-        <v>5830283.297821045</v>
+        <v>5510976.213912964</v>
       </c>
       <c r="G135" t="n">
-        <v>0.5814918538566606</v>
+        <v>0.5564138777866089</v>
       </c>
       <c r="H135" t="n">
-        <v>15.38649233473598</v>
+        <v>15.12214828476894</v>
       </c>
       <c r="I135" t="n">
-        <v>3.922561960598708</v>
+        <v>3.888720648846988</v>
       </c>
     </row>
     <row r="136">
@@ -4639,25 +4639,25 @@
         <v>825</v>
       </c>
       <c r="C136" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D136" t="n">
-        <v>-52.16448974609375</v>
+        <v>-57.33427429199219</v>
       </c>
       <c r="E136" t="n">
-        <v>60.96000671386719</v>
+        <v>64.4208984375</v>
       </c>
       <c r="F136" t="n">
-        <v>5679253.127593994</v>
+        <v>5350445.757858276</v>
       </c>
       <c r="G136" t="n">
-        <v>0.5664286383682402</v>
+        <v>0.540205973762137</v>
       </c>
       <c r="H136" t="n">
-        <v>15.23839565059458</v>
+        <v>15.01834188021675</v>
       </c>
       <c r="I136" t="n">
-        <v>3.903638770505614</v>
+        <v>3.875350549333151</v>
       </c>
     </row>
     <row r="137">
@@ -4670,25 +4670,25 @@
         <v>800</v>
       </c>
       <c r="C137" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D137" t="n">
-        <v>-50.418212890625</v>
+        <v>-56.57296752929688</v>
       </c>
       <c r="E137" t="n">
-        <v>60.94770812988281</v>
+        <v>62.50079345703125</v>
       </c>
       <c r="F137" t="n">
-        <v>5515778.191925049</v>
+        <v>5195667.209335327</v>
       </c>
       <c r="G137" t="n">
-        <v>0.5501242259502781</v>
+        <v>0.5245788091657099</v>
       </c>
       <c r="H137" t="n">
-        <v>15.21273498515589</v>
+        <v>15.05579209600858</v>
       </c>
       <c r="I137" t="n">
-        <v>3.900350623361429</v>
+        <v>3.880179389668548</v>
       </c>
     </row>
     <row r="138">
@@ -4701,25 +4701,25 @@
         <v>775</v>
       </c>
       <c r="C138" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D138" t="n">
-        <v>-49.16567993164062</v>
+        <v>-55.9935302734375</v>
       </c>
       <c r="E138" t="n">
-        <v>60.76625061035156</v>
+        <v>60.65386962890625</v>
       </c>
       <c r="F138" t="n">
-        <v>5309552.364990234</v>
+        <v>5040895.727371216</v>
       </c>
       <c r="G138" t="n">
-        <v>0.5295559907047843</v>
+        <v>0.5089523580420352</v>
       </c>
       <c r="H138" t="n">
-        <v>15.29012520552146</v>
+        <v>15.19906026417564</v>
       </c>
       <c r="I138" t="n">
-        <v>3.910258969112079</v>
+        <v>3.898597217484212</v>
       </c>
     </row>
     <row r="139">
@@ -4732,25 +4732,25 @@
         <v>750</v>
       </c>
       <c r="C139" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D139" t="n">
-        <v>-48.96044921875</v>
+        <v>-54.71180725097656</v>
       </c>
       <c r="E139" t="n">
-        <v>59.72929382324219</v>
+        <v>60.21696472167969</v>
       </c>
       <c r="F139" t="n">
-        <v>5056341.021194458</v>
+        <v>4870023.809310913</v>
       </c>
       <c r="G139" t="n">
-        <v>0.5043015860386549</v>
+        <v>0.4917003317508046</v>
       </c>
       <c r="H139" t="n">
-        <v>15.47025486413227</v>
+        <v>15.43317483305329</v>
       </c>
       <c r="I139" t="n">
-        <v>3.933224486872351</v>
+        <v>3.928507965252621</v>
       </c>
     </row>
     <row r="140">
@@ -4763,25 +4763,25 @@
         <v>725</v>
       </c>
       <c r="C140" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D140" t="n">
-        <v>-48.434814453125</v>
+        <v>-50.73023986816406</v>
       </c>
       <c r="E140" t="n">
-        <v>56.40139770507812</v>
+        <v>59.89950561523438</v>
       </c>
       <c r="F140" t="n">
-        <v>4489154.588195801</v>
+        <v>4468144.072311401</v>
       </c>
       <c r="G140" t="n">
-        <v>0.4477324154582145</v>
+        <v>0.4511246779667738</v>
       </c>
       <c r="H140" t="n">
-        <v>16.15148017788225</v>
+        <v>16.1600652836442</v>
       </c>
       <c r="I140" t="n">
-        <v>4.018890416256986</v>
+        <v>4.019958368396892</v>
       </c>
     </row>
     <row r="141">
@@ -4794,25 +4794,25 @@
         <v>700</v>
       </c>
       <c r="C141" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D141" t="n">
-        <v>-45.97933959960938</v>
+        <v>-45.50639343261719</v>
       </c>
       <c r="E141" t="n">
-        <v>54.9803466796875</v>
+        <v>58.38702392578125</v>
       </c>
       <c r="F141" t="n">
-        <v>3944211.800079346</v>
+        <v>4015814.099975586</v>
       </c>
       <c r="G141" t="n">
-        <v>0.3933817474167355</v>
+        <v>0.405455332976482</v>
       </c>
       <c r="H141" t="n">
-        <v>17.14517794723772</v>
+        <v>17.17154041476632</v>
       </c>
       <c r="I141" t="n">
-        <v>4.140673610324498</v>
+        <v>4.143855742514007</v>
       </c>
     </row>
     <row r="142">
@@ -4825,25 +4825,25 @@
         <v>650</v>
       </c>
       <c r="C142" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D142" t="n">
-        <v>-46.01249694824219</v>
+        <v>-43.6400146484375</v>
       </c>
       <c r="E142" t="n">
-        <v>53.02639770507812</v>
+        <v>56.6099853515625</v>
       </c>
       <c r="F142" t="n">
-        <v>3028931.376663208</v>
+        <v>3096296.016693115</v>
       </c>
       <c r="G142" t="n">
-        <v>0.3020949122796049</v>
+        <v>0.3126164959801551</v>
       </c>
       <c r="H142" t="n">
-        <v>17.99249601527588</v>
+        <v>17.99134883299492</v>
       </c>
       <c r="I142" t="n">
-        <v>4.241756241850288</v>
+        <v>4.241621014776652</v>
       </c>
     </row>
     <row r="143">
@@ -4856,25 +4856,25 @@
         <v>600</v>
       </c>
       <c r="C143" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D143" t="n">
-        <v>-45.54269409179688</v>
+        <v>-43.83694458007812</v>
       </c>
       <c r="E143" t="n">
-        <v>51.60366821289062</v>
+        <v>54.10940551757812</v>
       </c>
       <c r="F143" t="n">
-        <v>1591780.694747925</v>
+        <v>1683393.780944824</v>
       </c>
       <c r="G143" t="n">
-        <v>0.1587585816744345</v>
+        <v>0.1699632923714456</v>
       </c>
       <c r="H143" t="n">
-        <v>18.90006331741872</v>
+        <v>18.88071287889355</v>
       </c>
       <c r="I143" t="n">
-        <v>4.347420306045726</v>
+        <v>4.345194227982628</v>
       </c>
     </row>
     <row r="144">
@@ -4887,25 +4887,25 @@
         <v>550</v>
       </c>
       <c r="C144" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D144" t="n">
         <v>-46.11848449707031</v>
       </c>
       <c r="E144" t="n">
-        <v>53.69560241699219</v>
+        <v>51.68350219726562</v>
       </c>
       <c r="F144" t="n">
-        <v>646192.4318695068</v>
+        <v>876209.2996063232</v>
       </c>
       <c r="G144" t="n">
-        <v>0.06444894972708659</v>
+        <v>0.08846618007818947</v>
       </c>
       <c r="H144" t="n">
-        <v>20.68592604502885</v>
+        <v>20.73150990335025</v>
       </c>
       <c r="I144" t="n">
-        <v>4.548178321595235</v>
+        <v>4.553186785466884</v>
       </c>
     </row>
     <row r="145">
@@ -4918,25 +4918,25 @@
         <v>500</v>
       </c>
       <c r="C145" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D145" t="n">
-        <v>-52.96994018554688</v>
+        <v>-53.49273681640625</v>
       </c>
       <c r="E145" t="n">
-        <v>53.25816345214844</v>
+        <v>55.87313842773438</v>
       </c>
       <c r="F145" t="n">
-        <v>162560.3520812988</v>
+        <v>606624.3642425537</v>
       </c>
       <c r="G145" t="n">
-        <v>0.01621319508276266</v>
+        <v>0.06124762687523455</v>
       </c>
       <c r="H145" t="n">
-        <v>24.29358574198843</v>
+        <v>24.43359387259374</v>
       </c>
       <c r="I145" t="n">
-        <v>4.928852375755277</v>
+        <v>4.94303488482468</v>
       </c>
     </row>
     <row r="146">
@@ -4949,25 +4949,25 @@
         <v>450</v>
       </c>
       <c r="C146" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D146" t="n">
-        <v>-59.32827758789062</v>
+        <v>-60.30949401855469</v>
       </c>
       <c r="E146" t="n">
-        <v>62.3621826171875</v>
+        <v>60.88302612304688</v>
       </c>
       <c r="F146" t="n">
-        <v>-199866.6874542236</v>
+        <v>442040.8657684326</v>
       </c>
       <c r="G146" t="n">
-        <v>-0.01993399714476679</v>
+        <v>0.04463050877291382</v>
       </c>
       <c r="H146" t="n">
-        <v>30.29919735649806</v>
+        <v>30.59825982524179</v>
       </c>
       <c r="I146" t="n">
-        <v>5.504470669964375</v>
+        <v>5.531569381761544</v>
       </c>
     </row>
     <row r="147">
@@ -4980,25 +4980,25 @@
         <v>400</v>
       </c>
       <c r="C147" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D147" t="n">
-        <v>-64.51643371582031</v>
+        <v>-65.55380249023438</v>
       </c>
       <c r="E147" t="n">
-        <v>67.37187194824219</v>
+        <v>69.10142517089844</v>
       </c>
       <c r="F147" t="n">
-        <v>-1999696.746002197</v>
+        <v>-1297944.910583496</v>
       </c>
       <c r="G147" t="n">
-        <v>-0.1994426871878628</v>
+        <v>-0.1310465755645817</v>
       </c>
       <c r="H147" t="n">
-        <v>39.49901982341642</v>
+        <v>39.86690231730142</v>
       </c>
       <c r="I147" t="n">
-        <v>6.284824565842424</v>
+        <v>6.314024256945915</v>
       </c>
     </row>
     <row r="148">
@@ -5011,25 +5011,25 @@
         <v>350</v>
       </c>
       <c r="C148" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D148" t="n">
-        <v>-73.39028930664062</v>
+        <v>-68.04991149902344</v>
       </c>
       <c r="E148" t="n">
-        <v>71.73358154296875</v>
+        <v>75.79129028320312</v>
       </c>
       <c r="F148" t="n">
-        <v>-5368325.766494751</v>
+        <v>-4485034.063308716</v>
       </c>
       <c r="G148" t="n">
-        <v>-0.5354178420853304</v>
+        <v>-0.4528299702819311</v>
       </c>
       <c r="H148" t="n">
-        <v>53.91605239840818</v>
+        <v>54.34302113850518</v>
       </c>
       <c r="I148" t="n">
-        <v>7.342755095902912</v>
+        <v>7.371771913082036</v>
       </c>
     </row>
     <row r="149">
@@ -5042,25 +5042,25 @@
         <v>300</v>
       </c>
       <c r="C149" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D149" t="n">
-        <v>-70.07968139648438</v>
+        <v>-75.88917541503906</v>
       </c>
       <c r="E149" t="n">
-        <v>72.16477966308594</v>
+        <v>76.22332763671875</v>
       </c>
       <c r="F149" t="n">
-        <v>-8161206.19102478</v>
+        <v>-7393021.889068604</v>
       </c>
       <c r="G149" t="n">
-        <v>-0.8139698665241614</v>
+        <v>-0.7464339924880878</v>
       </c>
       <c r="H149" t="n">
-        <v>73.40046996390346</v>
+        <v>74.46044016084734</v>
       </c>
       <c r="I149" t="n">
-        <v>8.567407423713632</v>
+        <v>8.629046306565247</v>
       </c>
     </row>
     <row r="150">
@@ -5073,25 +5073,25 @@
         <v>250</v>
       </c>
       <c r="C150" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D150" t="n">
-        <v>-74.46308898925781</v>
+        <v>-75.75390625</v>
       </c>
       <c r="E150" t="n">
-        <v>71.28730773925781</v>
+        <v>76.65879821777344</v>
       </c>
       <c r="F150" t="n">
-        <v>-8586156.153442383</v>
+        <v>-7878754.465148926</v>
       </c>
       <c r="G150" t="n">
-        <v>-0.8563528741448863</v>
+        <v>-0.7954758202393685</v>
       </c>
       <c r="H150" t="n">
-        <v>81.41272557321636</v>
+        <v>82.81196684952947</v>
       </c>
       <c r="I150" t="n">
-        <v>9.022900064459119</v>
+        <v>9.100108068013778</v>
       </c>
     </row>
     <row r="151">
@@ -5104,25 +5104,25 @@
         <v>200</v>
       </c>
       <c r="C151" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D151" t="n">
-        <v>-67.33631896972656</v>
+        <v>-73.10708618164062</v>
       </c>
       <c r="E151" t="n">
-        <v>68.48300170898438</v>
+        <v>73.15193176269531</v>
       </c>
       <c r="F151" t="n">
-        <v>-8565346.925323486</v>
+        <v>-7850755.585342407</v>
       </c>
       <c r="G151" t="n">
-        <v>-0.8542774352651464</v>
+        <v>-0.7926489226658529</v>
       </c>
       <c r="H151" t="n">
-        <v>83.22094461297077</v>
+        <v>84.7807729290198</v>
       </c>
       <c r="I151" t="n">
-        <v>9.122551431094854</v>
+        <v>9.207647524151856</v>
       </c>
     </row>
     <row r="152">
@@ -5135,25 +5135,25 @@
         <v>150</v>
       </c>
       <c r="C152" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D152" t="n">
-        <v>-58.65924072265625</v>
+        <v>-67.24429321289062</v>
       </c>
       <c r="E152" t="n">
-        <v>59.37025451660156</v>
+        <v>68.32243347167969</v>
       </c>
       <c r="F152" t="n">
-        <v>-8425962.950408936</v>
+        <v>-7648084.759048462</v>
       </c>
       <c r="G152" t="n">
-        <v>-0.8403757701434471</v>
+        <v>-0.7721863301967119</v>
       </c>
       <c r="H152" t="n">
-        <v>75.16175704335838</v>
+        <v>76.23530081738039</v>
       </c>
       <c r="I152" t="n">
-        <v>8.669588054997675</v>
+        <v>8.731282884970593</v>
       </c>
     </row>
     <row r="153">
@@ -5166,25 +5166,25 @@
         <v>100</v>
       </c>
       <c r="C153" t="n">
-        <v>10026423</v>
+        <v>9904455</v>
       </c>
       <c r="D153" t="n">
-        <v>-55.7503662109375</v>
+        <v>-56.85836791992188</v>
       </c>
       <c r="E153" t="n">
-        <v>46.62557983398438</v>
+        <v>53.3455810546875</v>
       </c>
       <c r="F153" t="n">
-        <v>-7540293.468109131</v>
+        <v>-6530851.576309204</v>
       </c>
       <c r="G153" t="n">
-        <v>-0.7520422256381086</v>
+        <v>-0.6593852540406531</v>
       </c>
       <c r="H153" t="n">
-        <v>57.84846532460295</v>
+        <v>58.35943216376103</v>
       </c>
       <c r="I153" t="n">
-        <v>7.605817860335794</v>
+        <v>7.639334536709401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>